<commit_message>
Refresh player workbook veteran skills
</commit_message>
<xml_diff>
--- a/台灣籃球_球員完整資料.xlsx
+++ b/台灣籃球_球員完整資料.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="球員總表" sheetId="1" r:id="R6f3d4cb036aa47f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="2" r:id="R64e71d0c2aa34185"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="球員總表" sheetId="1" r:id="Re7a264c75cc4471b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="2" r:id="R527261444b4c43cc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11576,10 +11576,10 @@
         <x:v>800</x:v>
       </x:c>
       <x:c r="J281" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K281" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L281" s="22" t="str"/>
       <x:c r="M281" s="24" t="str"/>
@@ -11611,10 +11611,10 @@
         <x:v>750</x:v>
       </x:c>
       <x:c r="J282" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K282" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L282" s="22" t="str"/>
       <x:c r="M282" s="24" t="str"/>
@@ -11644,10 +11644,10 @@
         <x:v>1000</x:v>
       </x:c>
       <x:c r="J283" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K283" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L283" s="22" t="str"/>
       <x:c r="M283" s="24" t="str"/>
@@ -11677,10 +11677,10 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="J284" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K284" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L284" s="22" t="str"/>
       <x:c r="M284" s="24" t="str"/>
@@ -11710,10 +11710,10 @@
         <x:v>520</x:v>
       </x:c>
       <x:c r="J285" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K285" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L285" s="22" t="str"/>
       <x:c r="M285" s="24" t="str"/>
@@ -11743,10 +11743,10 @@
         <x:v>850</x:v>
       </x:c>
       <x:c r="J286" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K286" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L286" s="22" t="str"/>
       <x:c r="M286" s="24" t="str"/>
@@ -11776,10 +11776,10 @@
         <x:v>480</x:v>
       </x:c>
       <x:c r="J287" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K287" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L287" s="22" t="str"/>
       <x:c r="M287" s="24" t="str"/>
@@ -11809,10 +11809,10 @@
         <x:v>450</x:v>
       </x:c>
       <x:c r="J288" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K288" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L288" s="22" t="str"/>
       <x:c r="M288" s="24" t="str"/>
@@ -11844,10 +11844,10 @@
         <x:v>420</x:v>
       </x:c>
       <x:c r="J289" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K289" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L289" s="22" t="str"/>
       <x:c r="M289" s="24" t="str"/>
@@ -11877,10 +11877,10 @@
         <x:v>380</x:v>
       </x:c>
       <x:c r="J290" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K290" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L290" s="22" t="str"/>
       <x:c r="M290" s="24" t="str"/>
@@ -11912,10 +11912,10 @@
         <x:v>360</x:v>
       </x:c>
       <x:c r="J291" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K291" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L291" s="22" t="str"/>
       <x:c r="M291" s="24" t="str"/>
@@ -11945,10 +11945,10 @@
         <x:v>350</x:v>
       </x:c>
       <x:c r="J292" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K292" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L292" s="22" t="str"/>
       <x:c r="M292" s="24" t="str"/>
@@ -11978,10 +11978,10 @@
         <x:v>340</x:v>
       </x:c>
       <x:c r="J293" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K293" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L293" s="22" t="str"/>
       <x:c r="M293" s="24" t="str"/>
@@ -12011,10 +12011,10 @@
         <x:v>320</x:v>
       </x:c>
       <x:c r="J294" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K294" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L294" s="22" t="str"/>
       <x:c r="M294" s="24" t="str"/>
@@ -12044,10 +12044,10 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="J295" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K295" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L295" s="22" t="str"/>
       <x:c r="M295" s="24" t="str"/>
@@ -12077,10 +12077,10 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="J296" s="22" t="str">
-        <x:v>即戰力</x:v>
+        <x:v>老將領導</x:v>
       </x:c>
       <x:c r="K296" s="22" t="str">
-        <x:v>沒有特殊技能。</x:v>
+        <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
       <x:c r="L296" s="22" t="str"/>
       <x:c r="M296" s="24" t="str"/>
@@ -13678,7 +13678,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refd9de82eb304a57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5901d6c69b44486"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete veteran position catalog
</commit_message>
<xml_diff>
--- a/台灣籃球_球員完整資料.xlsx
+++ b/台灣籃球_球員完整資料.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="球員總表" sheetId="1" r:id="Re7a264c75cc4471b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="2" r:id="R527261444b4c43cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="球員總表" sheetId="1" r:id="Rdf40646bc5d9410f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="2" r:id="Rd8f83bc8e95a48f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11562,7 +11562,9 @@
       <x:c r="D281" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E281" s="22" t="str"/>
+      <x:c r="E281" s="22" t="str">
+        <x:v>SF/SG</x:v>
+      </x:c>
       <x:c r="F281" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -11630,7 +11632,9 @@
       <x:c r="D283" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E283" s="22" t="str"/>
+      <x:c r="E283" s="22" t="str">
+        <x:v>SF/SG</x:v>
+      </x:c>
       <x:c r="F283" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -11663,7 +11667,9 @@
       <x:c r="D284" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E284" s="22" t="str"/>
+      <x:c r="E284" s="22" t="str">
+        <x:v>C/PF</x:v>
+      </x:c>
       <x:c r="F284" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -11696,7 +11702,9 @@
       <x:c r="D285" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E285" s="22" t="str"/>
+      <x:c r="E285" s="22" t="str">
+        <x:v>C/PF</x:v>
+      </x:c>
       <x:c r="F285" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -11729,7 +11737,9 @@
       <x:c r="D286" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E286" s="22" t="str"/>
+      <x:c r="E286" s="22" t="str">
+        <x:v>SF/SG</x:v>
+      </x:c>
       <x:c r="F286" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -11762,7 +11772,9 @@
       <x:c r="D287" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E287" s="22" t="str"/>
+      <x:c r="E287" s="22" t="str">
+        <x:v>SF/PF</x:v>
+      </x:c>
       <x:c r="F287" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -11795,7 +11807,9 @@
       <x:c r="D288" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E288" s="22" t="str"/>
+      <x:c r="E288" s="22" t="str">
+        <x:v>SG/SF</x:v>
+      </x:c>
       <x:c r="F288" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -11863,7 +11877,9 @@
       <x:c r="D290" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E290" s="22" t="str"/>
+      <x:c r="E290" s="22" t="str">
+        <x:v>PF/C</x:v>
+      </x:c>
       <x:c r="F290" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -11931,7 +11947,9 @@
       <x:c r="D292" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E292" s="22" t="str"/>
+      <x:c r="E292" s="22" t="str">
+        <x:v>PG</x:v>
+      </x:c>
       <x:c r="F292" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -11964,7 +11982,9 @@
       <x:c r="D293" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E293" s="22" t="str"/>
+      <x:c r="E293" s="22" t="str">
+        <x:v>SF</x:v>
+      </x:c>
       <x:c r="F293" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -11997,7 +12017,9 @@
       <x:c r="D294" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E294" s="22" t="str"/>
+      <x:c r="E294" s="22" t="str">
+        <x:v>SG/SF</x:v>
+      </x:c>
       <x:c r="F294" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12030,7 +12052,9 @@
       <x:c r="D295" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E295" s="22" t="str"/>
+      <x:c r="E295" s="22" t="str">
+        <x:v>PG</x:v>
+      </x:c>
       <x:c r="F295" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12063,7 +12087,9 @@
       <x:c r="D296" s="22" t="str">
         <x:v>黃金世代資料</x:v>
       </x:c>
-      <x:c r="E296" s="22" t="str"/>
+      <x:c r="E296" s="22" t="str">
+        <x:v>PG</x:v>
+      </x:c>
       <x:c r="F296" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13678,7 +13704,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5901d6c69b44486"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7c4720733404326"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Sync player ratings from updated spreadsheet
</commit_message>
<xml_diff>
--- a/台灣籃球_球員完整資料.xlsx
+++ b/台灣籃球_球員完整資料.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="球員總表" sheetId="1" r:id="R63cd902fe70a471f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="2" r:id="Rf563120874714d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="球員總表" sheetId="1" r:id="R3fe57a073bc7479f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="2" r:id="Re9b8d4bbca714951"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -564,7 +564,7 @@
       <x:c r="K2" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L2" s="22"/>
+      <x:c r="L2" s="22" t="str"/>
       <x:c r="M2" s="24" t="str">
         <x:v>fubon_0</x:v>
       </x:c>
@@ -589,7 +589,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G3" s="23" t="n">
-        <x:v>70</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="H3" s="23" t="n">
         <x:v>76</x:v>
@@ -603,7 +603,7 @@
       <x:c r="K3" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L3" s="22"/>
+      <x:c r="L3" s="22" t="str"/>
       <x:c r="M3" s="24" t="str">
         <x:v>fubon_1</x:v>
       </x:c>
@@ -628,7 +628,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G4" s="23" t="n">
-        <x:v>85</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H4" s="23" t="n">
         <x:v>92</x:v>
@@ -642,7 +642,7 @@
       <x:c r="K4" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L4" s="22"/>
+      <x:c r="L4" s="22" t="str"/>
       <x:c r="M4" s="24" t="str">
         <x:v>fubon_2</x:v>
       </x:c>
@@ -681,7 +681,7 @@
       <x:c r="K5" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L5" s="22"/>
+      <x:c r="L5" s="22" t="str"/>
       <x:c r="M5" s="24" t="str">
         <x:v>fubon_3</x:v>
       </x:c>
@@ -720,7 +720,7 @@
       <x:c r="K6" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L6" s="22"/>
+      <x:c r="L6" s="22" t="str"/>
       <x:c r="M6" s="24" t="str">
         <x:v>fubon_4</x:v>
       </x:c>
@@ -759,7 +759,7 @@
       <x:c r="K7" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L7" s="22"/>
+      <x:c r="L7" s="22" t="str"/>
       <x:c r="M7" s="24" t="str">
         <x:v>fubon_5</x:v>
       </x:c>
@@ -798,7 +798,7 @@
       <x:c r="K8" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L8" s="22"/>
+      <x:c r="L8" s="22" t="str"/>
       <x:c r="M8" s="24" t="str">
         <x:v>fubon_6</x:v>
       </x:c>
@@ -837,7 +837,7 @@
       <x:c r="K9" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L9" s="22"/>
+      <x:c r="L9" s="22" t="str"/>
       <x:c r="M9" s="24" t="str">
         <x:v>fubon_7</x:v>
       </x:c>
@@ -876,7 +876,7 @@
       <x:c r="K10" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L10" s="22"/>
+      <x:c r="L10" s="22" t="str"/>
       <x:c r="M10" s="24" t="str">
         <x:v>fubon_8</x:v>
       </x:c>
@@ -915,7 +915,7 @@
       <x:c r="K11" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L11" s="22"/>
+      <x:c r="L11" s="22" t="str"/>
       <x:c r="M11" s="24" t="str">
         <x:v>fubon_9</x:v>
       </x:c>
@@ -1227,7 +1227,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G19" s="23" t="n">
-        <x:v>69</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="H19" s="23" t="n">
         <x:v>74</x:v>
@@ -1241,7 +1241,7 @@
       <x:c r="K19" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L19" s="22"/>
+      <x:c r="L19" s="22" t="str"/>
       <x:c r="M19" s="24" t="str">
         <x:v>pilots_0</x:v>
       </x:c>
@@ -1280,7 +1280,7 @@
       <x:c r="K20" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L20" s="22"/>
+      <x:c r="L20" s="22" t="str"/>
       <x:c r="M20" s="24" t="str">
         <x:v>pilots_1</x:v>
       </x:c>
@@ -1305,7 +1305,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G21" s="23" t="n">
-        <x:v>71</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="H21" s="23" t="n">
         <x:v>78</x:v>
@@ -1319,7 +1319,7 @@
       <x:c r="K21" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L21" s="22"/>
+      <x:c r="L21" s="22" t="str"/>
       <x:c r="M21" s="24" t="str">
         <x:v>pilots_2</x:v>
       </x:c>
@@ -1344,7 +1344,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G22" s="23" t="n">
-        <x:v>88</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="H22" s="23" t="n">
         <x:v>96</x:v>
@@ -1358,7 +1358,7 @@
       <x:c r="K22" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L22" s="22"/>
+      <x:c r="L22" s="22" t="str"/>
       <x:c r="M22" s="24" t="str">
         <x:v>pilots_3</x:v>
       </x:c>
@@ -1397,7 +1397,7 @@
       <x:c r="K23" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L23" s="22"/>
+      <x:c r="L23" s="22" t="str"/>
       <x:c r="M23" s="24" t="str">
         <x:v>pilots_4</x:v>
       </x:c>
@@ -1436,7 +1436,7 @@
       <x:c r="K24" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L24" s="22"/>
+      <x:c r="L24" s="22" t="str"/>
       <x:c r="M24" s="24" t="str">
         <x:v>pilots_5</x:v>
       </x:c>
@@ -1461,7 +1461,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G25" s="23" t="n">
-        <x:v>81</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="H25" s="23" t="n">
         <x:v>87</x:v>
@@ -1475,7 +1475,7 @@
       <x:c r="K25" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L25" s="22"/>
+      <x:c r="L25" s="22" t="str"/>
       <x:c r="M25" s="24" t="str">
         <x:v>pilots_6</x:v>
       </x:c>
@@ -1500,7 +1500,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G26" s="23" t="n">
-        <x:v>82</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H26" s="23" t="n">
         <x:v>89</x:v>
@@ -1514,7 +1514,7 @@
       <x:c r="K26" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L26" s="22"/>
+      <x:c r="L26" s="22" t="str"/>
       <x:c r="M26" s="24" t="str">
         <x:v>pilots_7</x:v>
       </x:c>
@@ -1539,7 +1539,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G27" s="23" t="n">
-        <x:v>83</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="H27" s="23" t="n">
         <x:v>91</x:v>
@@ -1553,7 +1553,7 @@
       <x:c r="K27" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L27" s="22"/>
+      <x:c r="L27" s="22" t="str"/>
       <x:c r="M27" s="24" t="str">
         <x:v>pilots_8</x:v>
       </x:c>
@@ -1592,7 +1592,7 @@
       <x:c r="K28" s="22" t="str">
         <x:v>輪替登場時提升活力與攻守連貫。</x:v>
       </x:c>
-      <x:c r="L28" s="22"/>
+      <x:c r="L28" s="22" t="str"/>
       <x:c r="M28" s="24" t="str">
         <x:v>pilots_9</x:v>
       </x:c>
@@ -1614,7 +1614,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="F29" s="22" t="str">
-        <x:v>local</x:v>
+        <x:v>foreign_student</x:v>
       </x:c>
       <x:c r="G29" s="23" t="n">
         <x:v>72</x:v>
@@ -1658,7 +1658,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G30" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H30" s="23" t="n">
         <x:v>79</x:v>
@@ -1713,7 +1713,7 @@
       <x:c r="K31" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L31" s="22"/>
+      <x:c r="L31" s="22" t="str"/>
       <x:c r="M31" s="24" t="str">
         <x:v>ghosthawks_0</x:v>
       </x:c>
@@ -1752,7 +1752,7 @@
       <x:c r="K32" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L32" s="22"/>
+      <x:c r="L32" s="22" t="str"/>
       <x:c r="M32" s="24" t="str">
         <x:v>ghosthawks_1</x:v>
       </x:c>
@@ -1791,7 +1791,7 @@
       <x:c r="K33" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L33" s="22"/>
+      <x:c r="L33" s="22" t="str"/>
       <x:c r="M33" s="24" t="str">
         <x:v>ghosthawks_3</x:v>
       </x:c>
@@ -1816,7 +1816,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G34" s="23" t="n">
-        <x:v>73</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="H34" s="23" t="n">
         <x:v>82</x:v>
@@ -1830,7 +1830,7 @@
       <x:c r="K34" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L34" s="22"/>
+      <x:c r="L34" s="22" t="str"/>
       <x:c r="M34" s="24" t="str">
         <x:v>ghosthawks_4</x:v>
       </x:c>
@@ -1869,7 +1869,7 @@
       <x:c r="K35" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L35" s="22"/>
+      <x:c r="L35" s="22" t="str"/>
       <x:c r="M35" s="24" t="str">
         <x:v>ghosthawks_5</x:v>
       </x:c>
@@ -1894,7 +1894,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G36" s="23" t="n">
-        <x:v>75</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H36" s="23" t="n">
         <x:v>81</x:v>
@@ -1908,7 +1908,7 @@
       <x:c r="K36" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L36" s="22"/>
+      <x:c r="L36" s="22" t="str"/>
       <x:c r="M36" s="24" t="str">
         <x:v>ghosthawks_6</x:v>
       </x:c>
@@ -1947,7 +1947,7 @@
       <x:c r="K37" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L37" s="22"/>
+      <x:c r="L37" s="22" t="str"/>
       <x:c r="M37" s="24" t="str">
         <x:v>ghosthawks_7</x:v>
       </x:c>
@@ -1986,7 +1986,7 @@
       <x:c r="K38" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L38" s="22"/>
+      <x:c r="L38" s="22" t="str"/>
       <x:c r="M38" s="24" t="str">
         <x:v>ghosthawks_8</x:v>
       </x:c>
@@ -2025,7 +2025,7 @@
       <x:c r="K39" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L39" s="22"/>
+      <x:c r="L39" s="22" t="str"/>
       <x:c r="M39" s="24" t="str">
         <x:v>ghosthawks_9</x:v>
       </x:c>
@@ -2050,7 +2050,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G40" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="H40" s="23" t="n">
         <x:v>79</x:v>
@@ -2091,7 +2091,7 @@
         <x:v>foreign_student</x:v>
       </x:c>
       <x:c r="G41" s="23" t="n">
-        <x:v>78</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="H41" s="23" t="n">
         <x:v>85</x:v>
@@ -2146,7 +2146,7 @@
       <x:c r="K42" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L42" s="22"/>
+      <x:c r="L42" s="22" t="str"/>
       <x:c r="M42" s="24" t="str">
         <x:v>yankey_0</x:v>
       </x:c>
@@ -2185,7 +2185,7 @@
       <x:c r="K43" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L43" s="22"/>
+      <x:c r="L43" s="22" t="str"/>
       <x:c r="M43" s="24" t="str">
         <x:v>yankey_1</x:v>
       </x:c>
@@ -2224,7 +2224,7 @@
       <x:c r="K44" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L44" s="22"/>
+      <x:c r="L44" s="22" t="str"/>
       <x:c r="M44" s="24" t="str">
         <x:v>yankey_2</x:v>
       </x:c>
@@ -2263,7 +2263,7 @@
       <x:c r="K45" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L45" s="22"/>
+      <x:c r="L45" s="22" t="str"/>
       <x:c r="M45" s="24" t="str">
         <x:v>yankey_3</x:v>
       </x:c>
@@ -2288,7 +2288,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G46" s="23" t="n">
-        <x:v>84</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="H46" s="23" t="n">
         <x:v>93</x:v>
@@ -2302,7 +2302,7 @@
       <x:c r="K46" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L46" s="22"/>
+      <x:c r="L46" s="22" t="str"/>
       <x:c r="M46" s="24" t="str">
         <x:v>yankey_4</x:v>
       </x:c>
@@ -2327,7 +2327,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G47" s="23" t="n">
-        <x:v>77</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="H47" s="23" t="n">
         <x:v>82</x:v>
@@ -2341,7 +2341,7 @@
       <x:c r="K47" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L47" s="22"/>
+      <x:c r="L47" s="22" t="str"/>
       <x:c r="M47" s="24" t="str">
         <x:v>yankey_5</x:v>
       </x:c>
@@ -2366,7 +2366,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G48" s="23" t="n">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="H48" s="23" t="n">
         <x:v>84</x:v>
@@ -2380,7 +2380,7 @@
       <x:c r="K48" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L48" s="22"/>
+      <x:c r="L48" s="22" t="str"/>
       <x:c r="M48" s="24" t="str">
         <x:v>yankey_6</x:v>
       </x:c>
@@ -2419,7 +2419,7 @@
       <x:c r="K49" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L49" s="22"/>
+      <x:c r="L49" s="22" t="str"/>
       <x:c r="M49" s="24" t="str">
         <x:v>yankey_7</x:v>
       </x:c>
@@ -2458,7 +2458,7 @@
       <x:c r="K50" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L50" s="22"/>
+      <x:c r="L50" s="22" t="str"/>
       <x:c r="M50" s="24" t="str">
         <x:v>yankey_8</x:v>
       </x:c>
@@ -2497,7 +2497,7 @@
       <x:c r="K51" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L51" s="22"/>
+      <x:c r="L51" s="22" t="str"/>
       <x:c r="M51" s="24" t="str">
         <x:v>yankey_9</x:v>
       </x:c>
@@ -2536,7 +2536,7 @@
       <x:c r="K52" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L52" s="22"/>
+      <x:c r="L52" s="22" t="str"/>
       <x:c r="M52" s="24" t="str">
         <x:v>yankey_10</x:v>
       </x:c>
@@ -2575,7 +2575,7 @@
       <x:c r="K53" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L53" s="22"/>
+      <x:c r="L53" s="22" t="str"/>
       <x:c r="M53" s="24" t="str">
         <x:v>yankey_11</x:v>
       </x:c>
@@ -2614,7 +2614,7 @@
       <x:c r="K54" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L54" s="22"/>
+      <x:c r="L54" s="22" t="str"/>
       <x:c r="M54" s="24" t="str">
         <x:v>yankey_12</x:v>
       </x:c>
@@ -2677,10 +2677,10 @@
         <x:v>PG/SG</x:v>
       </x:c>
       <x:c r="F56" s="22" t="str">
-        <x:v>local</x:v>
+        <x:v>foreign_student</x:v>
       </x:c>
       <x:c r="G56" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H56" s="23" t="n">
         <x:v>79</x:v>
@@ -2940,7 +2940,7 @@
       <x:c r="K62" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L62" s="22"/>
+      <x:c r="L62" s="22" t="str"/>
       <x:c r="M62" s="24" t="str">
         <x:v>dreamers_0</x:v>
       </x:c>
@@ -2959,13 +2959,13 @@
         <x:v>福爾摩沙夢想家</x:v>
       </x:c>
       <x:c r="E63" s="22" t="str">
-        <x:v>SF</x:v>
+        <x:v>SG/SF</x:v>
       </x:c>
       <x:c r="F63" s="22" t="str">
         <x:v>local</x:v>
       </x:c>
       <x:c r="G63" s="23" t="n">
-        <x:v>70</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H63" s="23" t="n">
         <x:v>76</x:v>
@@ -2979,7 +2979,7 @@
       <x:c r="K63" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L63" s="22"/>
+      <x:c r="L63" s="22" t="str"/>
       <x:c r="M63" s="24" t="str">
         <x:v>dreamers_1</x:v>
       </x:c>
@@ -3004,7 +3004,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G64" s="23" t="n">
-        <x:v>71</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="H64" s="23" t="n">
         <x:v>78</x:v>
@@ -3018,7 +3018,7 @@
       <x:c r="K64" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L64" s="22"/>
+      <x:c r="L64" s="22" t="str"/>
       <x:c r="M64" s="24" t="str">
         <x:v>dreamers_2</x:v>
       </x:c>
@@ -3043,7 +3043,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G65" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H65" s="23" t="n">
         <x:v>80</x:v>
@@ -3057,7 +3057,7 @@
       <x:c r="K65" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L65" s="22"/>
+      <x:c r="L65" s="22" t="str"/>
       <x:c r="M65" s="24" t="str">
         <x:v>dreamers_3</x:v>
       </x:c>
@@ -3082,7 +3082,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G66" s="23" t="n">
-        <x:v>84</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H66" s="23" t="n">
         <x:v>93</x:v>
@@ -3096,7 +3096,7 @@
       <x:c r="K66" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L66" s="22"/>
+      <x:c r="L66" s="22" t="str"/>
       <x:c r="M66" s="24" t="str">
         <x:v>dreamers_4</x:v>
       </x:c>
@@ -3121,7 +3121,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G67" s="23" t="n">
-        <x:v>83</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H67" s="23" t="n">
         <x:v>88</x:v>
@@ -3135,7 +3135,7 @@
       <x:c r="K67" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L67" s="22"/>
+      <x:c r="L67" s="22" t="str"/>
       <x:c r="M67" s="24" t="str">
         <x:v>dreamers_5</x:v>
       </x:c>
@@ -3160,7 +3160,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G68" s="23" t="n">
-        <x:v>75</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H68" s="23" t="n">
         <x:v>81</x:v>
@@ -3174,7 +3174,7 @@
       <x:c r="K68" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L68" s="22"/>
+      <x:c r="L68" s="22" t="str"/>
       <x:c r="M68" s="24" t="str">
         <x:v>dreamers_6</x:v>
       </x:c>
@@ -3213,7 +3213,7 @@
       <x:c r="K69" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L69" s="22"/>
+      <x:c r="L69" s="22" t="str"/>
       <x:c r="M69" s="24" t="str">
         <x:v>dreamers_7</x:v>
       </x:c>
@@ -3238,7 +3238,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G70" s="23" t="n">
-        <x:v>77</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H70" s="23" t="n">
         <x:v>85</x:v>
@@ -3252,7 +3252,7 @@
       <x:c r="K70" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L70" s="22"/>
+      <x:c r="L70" s="22" t="str"/>
       <x:c r="M70" s="24" t="str">
         <x:v>dreamers_8</x:v>
       </x:c>
@@ -3291,7 +3291,7 @@
       <x:c r="K71" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L71" s="22"/>
+      <x:c r="L71" s="22" t="str"/>
       <x:c r="M71" s="24" t="str">
         <x:v>dreamers_9</x:v>
       </x:c>
@@ -3330,7 +3330,7 @@
       <x:c r="K72" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L72" s="22"/>
+      <x:c r="L72" s="22" t="str"/>
       <x:c r="M72" s="24" t="str">
         <x:v>dreamers_10</x:v>
       </x:c>
@@ -3369,7 +3369,7 @@
       <x:c r="K73" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L73" s="22"/>
+      <x:c r="L73" s="22" t="str"/>
       <x:c r="M73" s="24" t="str">
         <x:v>dreamers_11</x:v>
       </x:c>
@@ -3394,7 +3394,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G74" s="23" t="n">
-        <x:v>85</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="H74" s="23" t="n">
         <x:v>92</x:v>
@@ -3408,7 +3408,7 @@
       <x:c r="K74" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L74" s="22"/>
+      <x:c r="L74" s="22" t="str"/>
       <x:c r="M74" s="24" t="str">
         <x:v>dreamers_12</x:v>
       </x:c>
@@ -3447,7 +3447,7 @@
       <x:c r="K75" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L75" s="22"/>
+      <x:c r="L75" s="22" t="str"/>
       <x:c r="M75" s="24" t="str">
         <x:v>dreamers_13</x:v>
       </x:c>
@@ -3609,7 +3609,7 @@
       <x:c r="K79" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L79" s="22"/>
+      <x:c r="L79" s="22" t="str"/>
       <x:c r="M79" s="24" t="str">
         <x:v>lioneers_0</x:v>
       </x:c>
@@ -3648,7 +3648,7 @@
       <x:c r="K80" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L80" s="22"/>
+      <x:c r="L80" s="22" t="str"/>
       <x:c r="M80" s="24" t="str">
         <x:v>lioneers_1</x:v>
       </x:c>
@@ -3687,7 +3687,7 @@
       <x:c r="K81" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L81" s="22"/>
+      <x:c r="L81" s="22" t="str"/>
       <x:c r="M81" s="24" t="str">
         <x:v>lioneers_2</x:v>
       </x:c>
@@ -3726,7 +3726,7 @@
       <x:c r="K82" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L82" s="22"/>
+      <x:c r="L82" s="22" t="str"/>
       <x:c r="M82" s="24" t="str">
         <x:v>lioneers_3</x:v>
       </x:c>
@@ -3765,7 +3765,7 @@
       <x:c r="K83" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L83" s="22"/>
+      <x:c r="L83" s="22" t="str"/>
       <x:c r="M83" s="24" t="str">
         <x:v>lioneers_4</x:v>
       </x:c>
@@ -3804,7 +3804,7 @@
       <x:c r="K84" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L84" s="22"/>
+      <x:c r="L84" s="22" t="str"/>
       <x:c r="M84" s="24" t="str">
         <x:v>lioneers_5</x:v>
       </x:c>
@@ -3829,7 +3829,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G85" s="23" t="n">
-        <x:v>75</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="H85" s="23" t="n">
         <x:v>81</x:v>
@@ -3843,7 +3843,7 @@
       <x:c r="K85" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L85" s="22"/>
+      <x:c r="L85" s="22" t="str"/>
       <x:c r="M85" s="24" t="str">
         <x:v>lioneers_6</x:v>
       </x:c>
@@ -3868,7 +3868,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G86" s="23" t="n">
-        <x:v>76</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="H86" s="23" t="n">
         <x:v>83</x:v>
@@ -3882,7 +3882,7 @@
       <x:c r="K86" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L86" s="22"/>
+      <x:c r="L86" s="22" t="str"/>
       <x:c r="M86" s="24" t="str">
         <x:v>lioneers_7</x:v>
       </x:c>
@@ -3921,7 +3921,7 @@
       <x:c r="K87" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L87" s="22"/>
+      <x:c r="L87" s="22" t="str"/>
       <x:c r="M87" s="24" t="str">
         <x:v>lioneers_8</x:v>
       </x:c>
@@ -3946,7 +3946,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G88" s="23" t="n">
-        <x:v>84</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H88" s="23" t="n">
         <x:v>93</x:v>
@@ -3960,7 +3960,7 @@
       <x:c r="K88" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L88" s="22"/>
+      <x:c r="L88" s="22" t="str"/>
       <x:c r="M88" s="24" t="str">
         <x:v>lioneers_9</x:v>
       </x:c>
@@ -3999,7 +3999,7 @@
       <x:c r="K89" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L89" s="22"/>
+      <x:c r="L89" s="22" t="str"/>
       <x:c r="M89" s="24" t="str">
         <x:v>lioneers_10</x:v>
       </x:c>
@@ -4038,7 +4038,7 @@
       <x:c r="K90" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L90" s="22"/>
+      <x:c r="L90" s="22" t="str"/>
       <x:c r="M90" s="24" t="str">
         <x:v>lioneers_11</x:v>
       </x:c>
@@ -4077,7 +4077,7 @@
       <x:c r="K91" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L91" s="22"/>
+      <x:c r="L91" s="22" t="str"/>
       <x:c r="M91" s="24" t="str">
         <x:v>lioneers_12</x:v>
       </x:c>
@@ -4116,7 +4116,7 @@
       <x:c r="K92" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L92" s="22"/>
+      <x:c r="L92" s="22" t="str"/>
       <x:c r="M92" s="24" t="str">
         <x:v>lioneers_13</x:v>
       </x:c>
@@ -4155,7 +4155,7 @@
       <x:c r="K93" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L93" s="22"/>
+      <x:c r="L93" s="22" t="str"/>
       <x:c r="M93" s="24" t="str">
         <x:v>lioneers_14</x:v>
       </x:c>
@@ -4194,7 +4194,7 @@
       <x:c r="K94" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L94" s="22"/>
+      <x:c r="L94" s="22" t="str"/>
       <x:c r="M94" s="24" t="str">
         <x:v>lioneers_15</x:v>
       </x:c>
@@ -4274,7 +4274,7 @@
       <x:c r="K96" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L96" s="22"/>
+      <x:c r="L96" s="22" t="str"/>
       <x:c r="M96" s="24" t="str">
         <x:v>aquas_0</x:v>
       </x:c>
@@ -4299,7 +4299,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G97" s="23" t="n">
-        <x:v>70</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H97" s="23" t="n">
         <x:v>76</x:v>
@@ -4313,7 +4313,7 @@
       <x:c r="K97" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L97" s="22"/>
+      <x:c r="L97" s="22" t="str"/>
       <x:c r="M97" s="24" t="str">
         <x:v>aquas_1</x:v>
       </x:c>
@@ -4352,7 +4352,7 @@
       <x:c r="K98" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L98" s="22"/>
+      <x:c r="L98" s="22" t="str"/>
       <x:c r="M98" s="24" t="str">
         <x:v>aquas_2</x:v>
       </x:c>
@@ -4391,7 +4391,7 @@
       <x:c r="K99" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L99" s="22"/>
+      <x:c r="L99" s="22" t="str"/>
       <x:c r="M99" s="24" t="str">
         <x:v>aquas_3</x:v>
       </x:c>
@@ -4430,7 +4430,7 @@
       <x:c r="K100" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L100" s="22"/>
+      <x:c r="L100" s="22" t="str"/>
       <x:c r="M100" s="24" t="str">
         <x:v>aquas_4</x:v>
       </x:c>
@@ -4469,7 +4469,7 @@
       <x:c r="K101" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L101" s="22"/>
+      <x:c r="L101" s="22" t="str"/>
       <x:c r="M101" s="24" t="str">
         <x:v>aquas_5</x:v>
       </x:c>
@@ -4508,7 +4508,7 @@
       <x:c r="K102" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L102" s="22"/>
+      <x:c r="L102" s="22" t="str"/>
       <x:c r="M102" s="24" t="str">
         <x:v>aquas_6</x:v>
       </x:c>
@@ -4547,7 +4547,7 @@
       <x:c r="K103" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L103" s="22"/>
+      <x:c r="L103" s="22" t="str"/>
       <x:c r="M103" s="24" t="str">
         <x:v>aquas_7</x:v>
       </x:c>
@@ -4586,7 +4586,7 @@
       <x:c r="K104" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L104" s="22"/>
+      <x:c r="L104" s="22" t="str"/>
       <x:c r="M104" s="24" t="str">
         <x:v>aquas_8</x:v>
       </x:c>
@@ -4611,7 +4611,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G105" s="23" t="n">
-        <x:v>84</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="H105" s="23" t="n">
         <x:v>93</x:v>
@@ -4625,7 +4625,7 @@
       <x:c r="K105" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L105" s="22"/>
+      <x:c r="L105" s="22" t="str"/>
       <x:c r="M105" s="24" t="str">
         <x:v>aquas_9</x:v>
       </x:c>
@@ -4664,7 +4664,7 @@
       <x:c r="K106" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L106" s="22"/>
+      <x:c r="L106" s="22" t="str"/>
       <x:c r="M106" s="24" t="str">
         <x:v>aquas_10</x:v>
       </x:c>
@@ -4703,7 +4703,7 @@
       <x:c r="K107" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L107" s="22"/>
+      <x:c r="L107" s="22" t="str"/>
       <x:c r="M107" s="24" t="str">
         <x:v>aquas_11</x:v>
       </x:c>
@@ -4742,7 +4742,7 @@
       <x:c r="K108" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L108" s="22"/>
+      <x:c r="L108" s="22" t="str"/>
       <x:c r="M108" s="24" t="str">
         <x:v>aquas_12</x:v>
       </x:c>
@@ -4781,7 +4781,7 @@
       <x:c r="K109" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L109" s="22"/>
+      <x:c r="L109" s="22" t="str"/>
       <x:c r="M109" s="24" t="str">
         <x:v>aquas_13</x:v>
       </x:c>
@@ -4888,7 +4888,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G112" s="23" t="n">
-        <x:v>88</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="H112" s="23" t="n">
         <x:v>93</x:v>
@@ -4902,7 +4902,7 @@
       <x:c r="K112" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L112" s="22"/>
+      <x:c r="L112" s="22" t="str"/>
       <x:c r="M112" s="24" t="str">
         <x:v>dea_0</x:v>
       </x:c>
@@ -4941,7 +4941,7 @@
       <x:c r="K113" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L113" s="22"/>
+      <x:c r="L113" s="22" t="str"/>
       <x:c r="M113" s="24" t="str">
         <x:v>dea_1</x:v>
       </x:c>
@@ -4980,7 +4980,7 @@
       <x:c r="K114" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L114" s="22"/>
+      <x:c r="L114" s="22" t="str"/>
       <x:c r="M114" s="24" t="str">
         <x:v>dea_2</x:v>
       </x:c>
@@ -5019,7 +5019,7 @@
       <x:c r="K115" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L115" s="22"/>
+      <x:c r="L115" s="22" t="str"/>
       <x:c r="M115" s="24" t="str">
         <x:v>dea_3</x:v>
       </x:c>
@@ -5058,7 +5058,7 @@
       <x:c r="K116" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L116" s="22"/>
+      <x:c r="L116" s="22" t="str"/>
       <x:c r="M116" s="24" t="str">
         <x:v>dea_4</x:v>
       </x:c>
@@ -5083,7 +5083,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G117" s="23" t="n">
-        <x:v>83</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H117" s="23" t="n">
         <x:v>88</x:v>
@@ -5097,7 +5097,7 @@
       <x:c r="K117" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L117" s="22"/>
+      <x:c r="L117" s="22" t="str"/>
       <x:c r="M117" s="24" t="str">
         <x:v>dea_5</x:v>
       </x:c>
@@ -5136,7 +5136,7 @@
       <x:c r="K118" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L118" s="22"/>
+      <x:c r="L118" s="22" t="str"/>
       <x:c r="M118" s="24" t="str">
         <x:v>dea_6</x:v>
       </x:c>
@@ -5175,7 +5175,7 @@
       <x:c r="K119" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L119" s="22"/>
+      <x:c r="L119" s="22" t="str"/>
       <x:c r="M119" s="24" t="str">
         <x:v>dea_7</x:v>
       </x:c>
@@ -5214,7 +5214,7 @@
       <x:c r="K120" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L120" s="22"/>
+      <x:c r="L120" s="22" t="str"/>
       <x:c r="M120" s="24" t="str">
         <x:v>dea_8</x:v>
       </x:c>
@@ -5253,7 +5253,7 @@
       <x:c r="K121" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L121" s="22"/>
+      <x:c r="L121" s="22" t="str"/>
       <x:c r="M121" s="24" t="str">
         <x:v>dea_9</x:v>
       </x:c>
@@ -5292,7 +5292,7 @@
       <x:c r="K122" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L122" s="22"/>
+      <x:c r="L122" s="22" t="str"/>
       <x:c r="M122" s="24" t="str">
         <x:v>dea_10</x:v>
       </x:c>
@@ -5317,7 +5317,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G123" s="23" t="n">
-        <x:v>70</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="H123" s="23" t="n">
         <x:v>76</x:v>
@@ -5331,7 +5331,7 @@
       <x:c r="K123" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L123" s="22"/>
+      <x:c r="L123" s="22" t="str"/>
       <x:c r="M123" s="24" t="str">
         <x:v>dea_11</x:v>
       </x:c>
@@ -5370,7 +5370,7 @@
       <x:c r="K124" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L124" s="22"/>
+      <x:c r="L124" s="22" t="str"/>
       <x:c r="M124" s="24" t="str">
         <x:v>dea_12</x:v>
       </x:c>
@@ -5409,7 +5409,7 @@
       <x:c r="K125" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L125" s="22"/>
+      <x:c r="L125" s="22" t="str"/>
       <x:c r="M125" s="24" t="str">
         <x:v>dea_13</x:v>
       </x:c>
@@ -5448,7 +5448,7 @@
       <x:c r="K126" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L126" s="22"/>
+      <x:c r="L126" s="22" t="str"/>
       <x:c r="M126" s="24" t="str">
         <x:v>dea_14</x:v>
       </x:c>
@@ -5555,7 +5555,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G129" s="23" t="n">
-        <x:v>85</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H129" s="23" t="n">
         <x:v>90</x:v>
@@ -5569,7 +5569,7 @@
       <x:c r="K129" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L129" s="22"/>
+      <x:c r="L129" s="22" t="str"/>
       <x:c r="M129" s="24" t="str">
         <x:v>kings_0</x:v>
       </x:c>
@@ -5608,7 +5608,7 @@
       <x:c r="K130" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L130" s="22"/>
+      <x:c r="L130" s="22" t="str"/>
       <x:c r="M130" s="24" t="str">
         <x:v>kings_1</x:v>
       </x:c>
@@ -5647,7 +5647,7 @@
       <x:c r="K131" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L131" s="22"/>
+      <x:c r="L131" s="22" t="str"/>
       <x:c r="M131" s="24" t="str">
         <x:v>kings_2</x:v>
       </x:c>
@@ -5686,7 +5686,7 @@
       <x:c r="K132" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L132" s="22"/>
+      <x:c r="L132" s="22" t="str"/>
       <x:c r="M132" s="24" t="str">
         <x:v>kings_3</x:v>
       </x:c>
@@ -5711,7 +5711,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G133" s="23" t="n">
-        <x:v>73</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="H133" s="23" t="n">
         <x:v>82</x:v>
@@ -5725,7 +5725,7 @@
       <x:c r="K133" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L133" s="22"/>
+      <x:c r="L133" s="22" t="str"/>
       <x:c r="M133" s="24" t="str">
         <x:v>kings_4</x:v>
       </x:c>
@@ -5764,7 +5764,7 @@
       <x:c r="K134" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L134" s="22"/>
+      <x:c r="L134" s="22" t="str"/>
       <x:c r="M134" s="24" t="str">
         <x:v>kings_5</x:v>
       </x:c>
@@ -5803,7 +5803,7 @@
       <x:c r="K135" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L135" s="22"/>
+      <x:c r="L135" s="22" t="str"/>
       <x:c r="M135" s="24" t="str">
         <x:v>kings_6</x:v>
       </x:c>
@@ -5842,7 +5842,7 @@
       <x:c r="K136" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L136" s="22"/>
+      <x:c r="L136" s="22" t="str"/>
       <x:c r="M136" s="24" t="str">
         <x:v>kings_7</x:v>
       </x:c>
@@ -5867,7 +5867,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G137" s="23" t="n">
-        <x:v>77</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H137" s="23" t="n">
         <x:v>85</x:v>
@@ -5881,7 +5881,7 @@
       <x:c r="K137" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L137" s="22"/>
+      <x:c r="L137" s="22" t="str"/>
       <x:c r="M137" s="24" t="str">
         <x:v>kings_8</x:v>
       </x:c>
@@ -5906,7 +5906,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G138" s="23" t="n">
-        <x:v>78</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="H138" s="23" t="n">
         <x:v>87</x:v>
@@ -5920,7 +5920,7 @@
       <x:c r="K138" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L138" s="22"/>
+      <x:c r="L138" s="22" t="str"/>
       <x:c r="M138" s="24" t="str">
         <x:v>kings_9</x:v>
       </x:c>
@@ -5945,7 +5945,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G139" s="23" t="n">
-        <x:v>69</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="H139" s="23" t="n">
         <x:v>74</x:v>
@@ -5959,7 +5959,7 @@
       <x:c r="K139" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L139" s="22"/>
+      <x:c r="L139" s="22" t="str"/>
       <x:c r="M139" s="24" t="str">
         <x:v>kings_10</x:v>
       </x:c>
@@ -5998,7 +5998,7 @@
       <x:c r="K140" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L140" s="22"/>
+      <x:c r="L140" s="22" t="str"/>
       <x:c r="M140" s="24" t="str">
         <x:v>kings_11</x:v>
       </x:c>
@@ -6037,7 +6037,7 @@
       <x:c r="K141" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L141" s="22"/>
+      <x:c r="L141" s="22" t="str"/>
       <x:c r="M141" s="24" t="str">
         <x:v>kings_12</x:v>
       </x:c>
@@ -6076,7 +6076,7 @@
       <x:c r="K142" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L142" s="22"/>
+      <x:c r="L142" s="22" t="str"/>
       <x:c r="M142" s="24" t="str">
         <x:v>kings_13</x:v>
       </x:c>
@@ -6115,7 +6115,7 @@
       <x:c r="K143" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L143" s="22"/>
+      <x:c r="L143" s="22" t="str"/>
       <x:c r="M143" s="24" t="str">
         <x:v>ghosthawks_2</x:v>
       </x:c>
@@ -6222,7 +6222,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G146" s="23" t="n">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="H146" s="23" t="n">
         <x:v>90</x:v>
@@ -6263,7 +6263,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G147" s="23" t="n">
-        <x:v>82</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H147" s="23" t="n">
         <x:v>89</x:v>
@@ -6345,7 +6345,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G149" s="23" t="n">
-        <x:v>85</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H149" s="23" t="n">
         <x:v>90</x:v>
@@ -6400,7 +6400,7 @@
       <x:c r="K150" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L150" s="22"/>
+      <x:c r="L150" s="22" t="str"/>
       <x:c r="M150" s="24" t="str">
         <x:v>mars_0</x:v>
       </x:c>
@@ -6439,7 +6439,7 @@
       <x:c r="K151" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L151" s="22"/>
+      <x:c r="L151" s="22" t="str"/>
       <x:c r="M151" s="24" t="str">
         <x:v>mars_1</x:v>
       </x:c>
@@ -6478,7 +6478,7 @@
       <x:c r="K152" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L152" s="22"/>
+      <x:c r="L152" s="22" t="str"/>
       <x:c r="M152" s="24" t="str">
         <x:v>mars_2</x:v>
       </x:c>
@@ -6517,7 +6517,7 @@
       <x:c r="K153" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L153" s="22"/>
+      <x:c r="L153" s="22" t="str"/>
       <x:c r="M153" s="24" t="str">
         <x:v>mars_3</x:v>
       </x:c>
@@ -6556,7 +6556,7 @@
       <x:c r="K154" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L154" s="22"/>
+      <x:c r="L154" s="22" t="str"/>
       <x:c r="M154" s="24" t="str">
         <x:v>mars_4</x:v>
       </x:c>
@@ -6595,7 +6595,7 @@
       <x:c r="K155" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L155" s="22"/>
+      <x:c r="L155" s="22" t="str"/>
       <x:c r="M155" s="24" t="str">
         <x:v>mars_5</x:v>
       </x:c>
@@ -6634,7 +6634,7 @@
       <x:c r="K156" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L156" s="22"/>
+      <x:c r="L156" s="22" t="str"/>
       <x:c r="M156" s="24" t="str">
         <x:v>mars_6</x:v>
       </x:c>
@@ -6673,7 +6673,7 @@
       <x:c r="K157" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L157" s="22"/>
+      <x:c r="L157" s="22" t="str"/>
       <x:c r="M157" s="24" t="str">
         <x:v>mars_7</x:v>
       </x:c>
@@ -6712,7 +6712,7 @@
       <x:c r="K158" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L158" s="22"/>
+      <x:c r="L158" s="22" t="str"/>
       <x:c r="M158" s="24" t="str">
         <x:v>mars_8</x:v>
       </x:c>
@@ -6737,7 +6737,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G159" s="23" t="n">
-        <x:v>84</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H159" s="23" t="n">
         <x:v>93</x:v>
@@ -6751,7 +6751,7 @@
       <x:c r="K159" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L159" s="22"/>
+      <x:c r="L159" s="22" t="str"/>
       <x:c r="M159" s="24" t="str">
         <x:v>mars_9</x:v>
       </x:c>
@@ -6776,7 +6776,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G160" s="23" t="n">
-        <x:v>69</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H160" s="23" t="n">
         <x:v>74</x:v>
@@ -6790,7 +6790,7 @@
       <x:c r="K160" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L160" s="22"/>
+      <x:c r="L160" s="22" t="str"/>
       <x:c r="M160" s="24" t="str">
         <x:v>mars_10</x:v>
       </x:c>
@@ -6829,7 +6829,7 @@
       <x:c r="K161" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L161" s="22"/>
+      <x:c r="L161" s="22" t="str"/>
       <x:c r="M161" s="24" t="str">
         <x:v>mars_11</x:v>
       </x:c>
@@ -6854,7 +6854,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G162" s="23" t="n">
-        <x:v>71</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="H162" s="23" t="n">
         <x:v>78</x:v>
@@ -6868,7 +6868,7 @@
       <x:c r="K162" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L162" s="22"/>
+      <x:c r="L162" s="22" t="str"/>
       <x:c r="M162" s="24" t="str">
         <x:v>mars_12</x:v>
       </x:c>
@@ -6934,7 +6934,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G164" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="H164" s="23" t="n">
         <x:v>79</x:v>
@@ -6975,7 +6975,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G165" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="H165" s="23" t="n">
         <x:v>79</x:v>
@@ -7071,7 +7071,7 @@
       <x:c r="K167" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L167" s="22"/>
+      <x:c r="L167" s="22" t="str"/>
       <x:c r="M167" s="24" t="str">
         <x:v>leopards_0</x:v>
       </x:c>
@@ -7096,7 +7096,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G168" s="23" t="n">
-        <x:v>85</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H168" s="23" t="n">
         <x:v>91</x:v>
@@ -7110,7 +7110,7 @@
       <x:c r="K168" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L168" s="22"/>
+      <x:c r="L168" s="22" t="str"/>
       <x:c r="M168" s="24" t="str">
         <x:v>leopards_1</x:v>
       </x:c>
@@ -7149,7 +7149,7 @@
       <x:c r="K169" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L169" s="22"/>
+      <x:c r="L169" s="22" t="str"/>
       <x:c r="M169" s="24" t="str">
         <x:v>leopards_2</x:v>
       </x:c>
@@ -7188,7 +7188,7 @@
       <x:c r="K170" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L170" s="22"/>
+      <x:c r="L170" s="22" t="str"/>
       <x:c r="M170" s="24" t="str">
         <x:v>leopards_3</x:v>
       </x:c>
@@ -7227,7 +7227,7 @@
       <x:c r="K171" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L171" s="22"/>
+      <x:c r="L171" s="22" t="str"/>
       <x:c r="M171" s="24" t="str">
         <x:v>leopards_4</x:v>
       </x:c>
@@ -7266,7 +7266,7 @@
       <x:c r="K172" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L172" s="22"/>
+      <x:c r="L172" s="22" t="str"/>
       <x:c r="M172" s="24" t="str">
         <x:v>leopards_5</x:v>
       </x:c>
@@ -7305,7 +7305,7 @@
       <x:c r="K173" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L173" s="22"/>
+      <x:c r="L173" s="22" t="str"/>
       <x:c r="M173" s="24" t="str">
         <x:v>leopards_6</x:v>
       </x:c>
@@ -7330,7 +7330,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G174" s="23" t="n">
-        <x:v>76</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="H174" s="23" t="n">
         <x:v>83</x:v>
@@ -7344,7 +7344,7 @@
       <x:c r="K174" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L174" s="22"/>
+      <x:c r="L174" s="22" t="str"/>
       <x:c r="M174" s="24" t="str">
         <x:v>leopards_7</x:v>
       </x:c>
@@ -7383,7 +7383,7 @@
       <x:c r="K175" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L175" s="22"/>
+      <x:c r="L175" s="22" t="str"/>
       <x:c r="M175" s="24" t="str">
         <x:v>leopards_8</x:v>
       </x:c>
@@ -7408,7 +7408,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G176" s="23" t="n">
-        <x:v>84</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H176" s="23" t="n">
         <x:v>93</x:v>
@@ -7422,7 +7422,7 @@
       <x:c r="K176" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L176" s="22"/>
+      <x:c r="L176" s="22" t="str"/>
       <x:c r="M176" s="24" t="str">
         <x:v>leopards_9</x:v>
       </x:c>
@@ -7461,7 +7461,7 @@
       <x:c r="K177" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L177" s="22"/>
+      <x:c r="L177" s="22" t="str"/>
       <x:c r="M177" s="24" t="str">
         <x:v>leopards_10</x:v>
       </x:c>
@@ -7486,7 +7486,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G178" s="23" t="n">
-        <x:v>70</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="H178" s="23" t="n">
         <x:v>76</x:v>
@@ -7500,7 +7500,7 @@
       <x:c r="K178" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L178" s="22"/>
+      <x:c r="L178" s="22" t="str"/>
       <x:c r="M178" s="24" t="str">
         <x:v>leopards_11</x:v>
       </x:c>
@@ -7525,7 +7525,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G179" s="23" t="n">
-        <x:v>71</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="H179" s="23" t="n">
         <x:v>78</x:v>
@@ -7539,7 +7539,7 @@
       <x:c r="K179" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L179" s="22"/>
+      <x:c r="L179" s="22" t="str"/>
       <x:c r="M179" s="24" t="str">
         <x:v>leopards_12</x:v>
       </x:c>
@@ -7578,7 +7578,7 @@
       <x:c r="K180" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L180" s="22"/>
+      <x:c r="L180" s="22" t="str"/>
       <x:c r="M180" s="24" t="str">
         <x:v>leopards_13</x:v>
       </x:c>
@@ -7740,7 +7740,7 @@
       <x:c r="K184" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L184" s="22"/>
+      <x:c r="L184" s="22" t="str"/>
       <x:c r="M184" s="24" t="str">
         <x:v>sbl_pure_0</x:v>
       </x:c>
@@ -7779,7 +7779,7 @@
       <x:c r="K185" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L185" s="22"/>
+      <x:c r="L185" s="22" t="str"/>
       <x:c r="M185" s="24" t="str">
         <x:v>sbl_pure_1</x:v>
       </x:c>
@@ -7818,7 +7818,7 @@
       <x:c r="K186" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L186" s="22"/>
+      <x:c r="L186" s="22" t="str"/>
       <x:c r="M186" s="24" t="str">
         <x:v>sbl_pure_2</x:v>
       </x:c>
@@ -7857,7 +7857,7 @@
       <x:c r="K187" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L187" s="22"/>
+      <x:c r="L187" s="22" t="str"/>
       <x:c r="M187" s="24" t="str">
         <x:v>sbl_pure_3</x:v>
       </x:c>
@@ -7882,7 +7882,7 @@
         <x:v>foreign_student</x:v>
       </x:c>
       <x:c r="G188" s="23" t="n">
-        <x:v>84</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="H188" s="23" t="n">
         <x:v>93</x:v>
@@ -7896,7 +7896,7 @@
       <x:c r="K188" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L188" s="22"/>
+      <x:c r="L188" s="22" t="str"/>
       <x:c r="M188" s="24" t="str">
         <x:v>sbl_pure_4</x:v>
       </x:c>
@@ -7935,7 +7935,7 @@
       <x:c r="K189" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L189" s="22"/>
+      <x:c r="L189" s="22" t="str"/>
       <x:c r="M189" s="24" t="str">
         <x:v>sbl_pure_5</x:v>
       </x:c>
@@ -7960,7 +7960,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G190" s="23" t="n">
-        <x:v>75</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="H190" s="23" t="n">
         <x:v>81</x:v>
@@ -7974,7 +7974,7 @@
       <x:c r="K190" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L190" s="22"/>
+      <x:c r="L190" s="22" t="str"/>
       <x:c r="M190" s="24" t="str">
         <x:v>sbl_pure_6</x:v>
       </x:c>
@@ -7999,7 +7999,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G191" s="23" t="n">
-        <x:v>76</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H191" s="23" t="n">
         <x:v>83</x:v>
@@ -8013,7 +8013,7 @@
       <x:c r="K191" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L191" s="22"/>
+      <x:c r="L191" s="22" t="str"/>
       <x:c r="M191" s="24" t="str">
         <x:v>sbl_pure_7</x:v>
       </x:c>
@@ -8038,7 +8038,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G192" s="23" t="n">
-        <x:v>77</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H192" s="23" t="n">
         <x:v>85</x:v>
@@ -8052,7 +8052,7 @@
       <x:c r="K192" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L192" s="22"/>
+      <x:c r="L192" s="22" t="str"/>
       <x:c r="M192" s="24" t="str">
         <x:v>sbl_pure_8</x:v>
       </x:c>
@@ -8091,7 +8091,7 @@
       <x:c r="K193" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L193" s="22"/>
+      <x:c r="L193" s="22" t="str"/>
       <x:c r="M193" s="24" t="str">
         <x:v>sbl_pure_9</x:v>
       </x:c>
@@ -8130,7 +8130,7 @@
       <x:c r="K194" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L194" s="22"/>
+      <x:c r="L194" s="22" t="str"/>
       <x:c r="M194" s="24" t="str">
         <x:v>sbl_pure_10</x:v>
       </x:c>
@@ -8374,7 +8374,7 @@
       <x:c r="K200" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L200" s="22"/>
+      <x:c r="L200" s="22" t="str"/>
       <x:c r="M200" s="24" t="str">
         <x:v>sbl_kites_0</x:v>
       </x:c>
@@ -8413,7 +8413,7 @@
       <x:c r="K201" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L201" s="22"/>
+      <x:c r="L201" s="22" t="str"/>
       <x:c r="M201" s="24" t="str">
         <x:v>sbl_kites_1</x:v>
       </x:c>
@@ -8452,7 +8452,7 @@
       <x:c r="K202" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L202" s="22"/>
+      <x:c r="L202" s="22" t="str"/>
       <x:c r="M202" s="24" t="str">
         <x:v>sbl_kites_2</x:v>
       </x:c>
@@ -8471,7 +8471,7 @@
         <x:v>基隆黑鳶</x:v>
       </x:c>
       <x:c r="E203" s="22" t="str">
-        <x:v>PG</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="F203" s="22" t="str">
         <x:v>local</x:v>
@@ -8491,7 +8491,7 @@
       <x:c r="K203" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L203" s="22"/>
+      <x:c r="L203" s="22" t="str"/>
       <x:c r="M203" s="24" t="str">
         <x:v>sbl_kites_3</x:v>
       </x:c>
@@ -8510,7 +8510,7 @@
         <x:v>基隆黑鳶</x:v>
       </x:c>
       <x:c r="E204" s="22" t="str">
-        <x:v>PG</x:v>
+        <x:v>SG</x:v>
       </x:c>
       <x:c r="F204" s="22" t="str">
         <x:v>local</x:v>
@@ -8530,7 +8530,7 @@
       <x:c r="K204" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L204" s="22"/>
+      <x:c r="L204" s="22" t="str"/>
       <x:c r="M204" s="24" t="str">
         <x:v>sbl_kites_5</x:v>
       </x:c>
@@ -8569,7 +8569,7 @@
       <x:c r="K205" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L205" s="22"/>
+      <x:c r="L205" s="22" t="str"/>
       <x:c r="M205" s="24" t="str">
         <x:v>sbl_kites_6</x:v>
       </x:c>
@@ -8588,13 +8588,13 @@
         <x:v>基隆黑鳶</x:v>
       </x:c>
       <x:c r="E206" s="22" t="str">
-        <x:v>SF</x:v>
+        <x:v>PF</x:v>
       </x:c>
       <x:c r="F206" s="22" t="str">
         <x:v>local</x:v>
       </x:c>
       <x:c r="G206" s="23" t="n">
-        <x:v>77</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="H206" s="23" t="n">
         <x:v>85</x:v>
@@ -8608,7 +8608,7 @@
       <x:c r="K206" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L206" s="22"/>
+      <x:c r="L206" s="22" t="str"/>
       <x:c r="M206" s="24" t="str">
         <x:v>sbl_kites_8</x:v>
       </x:c>
@@ -8633,7 +8633,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G207" s="23" t="n">
-        <x:v>78</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="H207" s="23" t="n">
         <x:v>87</x:v>
@@ -8647,7 +8647,7 @@
       <x:c r="K207" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L207" s="22"/>
+      <x:c r="L207" s="22" t="str"/>
       <x:c r="M207" s="24" t="str">
         <x:v>sbl_kites_9</x:v>
       </x:c>
@@ -8686,7 +8686,7 @@
       <x:c r="K208" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L208" s="22"/>
+      <x:c r="L208" s="22" t="str"/>
       <x:c r="M208" s="24" t="str">
         <x:v>sbl_kites_10</x:v>
       </x:c>
@@ -8930,7 +8930,7 @@
       <x:c r="K214" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L214" s="22"/>
+      <x:c r="L214" s="22" t="str"/>
       <x:c r="M214" s="24" t="str">
         <x:v>sbl_bank_0</x:v>
       </x:c>
@@ -8969,7 +8969,7 @@
       <x:c r="K215" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L215" s="22"/>
+      <x:c r="L215" s="22" t="str"/>
       <x:c r="M215" s="24" t="str">
         <x:v>sbl_bank_1</x:v>
       </x:c>
@@ -9008,7 +9008,7 @@
       <x:c r="K216" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L216" s="22"/>
+      <x:c r="L216" s="22" t="str"/>
       <x:c r="M216" s="24" t="str">
         <x:v>sbl_bank_2</x:v>
       </x:c>
@@ -9047,7 +9047,7 @@
       <x:c r="K217" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L217" s="22"/>
+      <x:c r="L217" s="22" t="str"/>
       <x:c r="M217" s="24" t="str">
         <x:v>sbl_bank_3</x:v>
       </x:c>
@@ -9086,7 +9086,7 @@
       <x:c r="K218" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L218" s="22"/>
+      <x:c r="L218" s="22" t="str"/>
       <x:c r="M218" s="24" t="str">
         <x:v>sbl_bank_4</x:v>
       </x:c>
@@ -9125,7 +9125,7 @@
       <x:c r="K219" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L219" s="22"/>
+      <x:c r="L219" s="22" t="str"/>
       <x:c r="M219" s="24" t="str">
         <x:v>sbl_bank_5</x:v>
       </x:c>
@@ -9144,7 +9144,7 @@
         <x:v>臺灣銀行</x:v>
       </x:c>
       <x:c r="E220" s="22" t="str">
-        <x:v>SF</x:v>
+        <x:v>SH/SF</x:v>
       </x:c>
       <x:c r="F220" s="22" t="str">
         <x:v>local</x:v>
@@ -9164,7 +9164,7 @@
       <x:c r="K220" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L220" s="22"/>
+      <x:c r="L220" s="22" t="str"/>
       <x:c r="M220" s="24" t="str">
         <x:v>sbl_bank_6</x:v>
       </x:c>
@@ -9189,7 +9189,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G221" s="23" t="n">
-        <x:v>76</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="H221" s="23" t="n">
         <x:v>83</x:v>
@@ -9203,7 +9203,7 @@
       <x:c r="K221" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L221" s="22"/>
+      <x:c r="L221" s="22" t="str"/>
       <x:c r="M221" s="24" t="str">
         <x:v>sbl_bank_7</x:v>
       </x:c>
@@ -9228,7 +9228,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G222" s="23" t="n">
-        <x:v>77</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H222" s="23" t="n">
         <x:v>85</x:v>
@@ -9242,7 +9242,7 @@
       <x:c r="K222" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L222" s="22"/>
+      <x:c r="L222" s="22" t="str"/>
       <x:c r="M222" s="24" t="str">
         <x:v>sbl_bank_8</x:v>
       </x:c>
@@ -9267,7 +9267,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G223" s="23" t="n">
-        <x:v>84</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H223" s="23" t="n">
         <x:v>93</x:v>
@@ -9281,7 +9281,7 @@
       <x:c r="K223" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L223" s="22"/>
+      <x:c r="L223" s="22" t="str"/>
       <x:c r="M223" s="24" t="str">
         <x:v>sbl_bank_9</x:v>
       </x:c>
@@ -9730,7 +9730,7 @@
       <x:c r="K234" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L234" s="22"/>
+      <x:c r="L234" s="22" t="str"/>
       <x:c r="M234" s="24" t="str">
         <x:v>sbl_beer_0</x:v>
       </x:c>
@@ -9769,7 +9769,7 @@
       <x:c r="K235" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L235" s="22"/>
+      <x:c r="L235" s="22" t="str"/>
       <x:c r="M235" s="24" t="str">
         <x:v>sbl_beer_1</x:v>
       </x:c>
@@ -9808,7 +9808,7 @@
       <x:c r="K236" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L236" s="22"/>
+      <x:c r="L236" s="22" t="str"/>
       <x:c r="M236" s="24" t="str">
         <x:v>sbl_beer_2</x:v>
       </x:c>
@@ -9833,7 +9833,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G237" s="23" t="n">
-        <x:v>83</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H237" s="23" t="n">
         <x:v>91</x:v>
@@ -9847,7 +9847,7 @@
       <x:c r="K237" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L237" s="22"/>
+      <x:c r="L237" s="22" t="str"/>
       <x:c r="M237" s="24" t="str">
         <x:v>sbl_beer_3</x:v>
       </x:c>
@@ -9872,7 +9872,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G238" s="23" t="n">
-        <x:v>73</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H238" s="23" t="n">
         <x:v>82</x:v>
@@ -9886,7 +9886,7 @@
       <x:c r="K238" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L238" s="22"/>
+      <x:c r="L238" s="22" t="str"/>
       <x:c r="M238" s="24" t="str">
         <x:v>sbl_beer_4</x:v>
       </x:c>
@@ -9925,7 +9925,7 @@
       <x:c r="K239" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L239" s="22"/>
+      <x:c r="L239" s="22" t="str"/>
       <x:c r="M239" s="24" t="str">
         <x:v>sbl_beer_5</x:v>
       </x:c>
@@ -9950,7 +9950,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G240" s="23" t="n">
-        <x:v>75</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H240" s="23" t="n">
         <x:v>81</x:v>
@@ -9964,7 +9964,7 @@
       <x:c r="K240" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L240" s="22"/>
+      <x:c r="L240" s="22" t="str"/>
       <x:c r="M240" s="24" t="str">
         <x:v>sbl_beer_6</x:v>
       </x:c>
@@ -9989,7 +9989,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G241" s="23" t="n">
-        <x:v>76</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="H241" s="23" t="n">
         <x:v>83</x:v>
@@ -10003,7 +10003,7 @@
       <x:c r="K241" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L241" s="22"/>
+      <x:c r="L241" s="22" t="str"/>
       <x:c r="M241" s="24" t="str">
         <x:v>sbl_beer_7</x:v>
       </x:c>
@@ -10028,7 +10028,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G242" s="23" t="n">
-        <x:v>77</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H242" s="23" t="n">
         <x:v>85</x:v>
@@ -10042,7 +10042,7 @@
       <x:c r="K242" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L242" s="22"/>
+      <x:c r="L242" s="22" t="str"/>
       <x:c r="M242" s="24" t="str">
         <x:v>sbl_beer_8</x:v>
       </x:c>
@@ -10067,7 +10067,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G243" s="23" t="n">
-        <x:v>78</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="H243" s="23" t="n">
         <x:v>87</x:v>
@@ -10081,7 +10081,7 @@
       <x:c r="K243" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L243" s="22"/>
+      <x:c r="L243" s="22" t="str"/>
       <x:c r="M243" s="24" t="str">
         <x:v>sbl_beer_9</x:v>
       </x:c>
@@ -10106,7 +10106,7 @@
         <x:v>foreign_student</x:v>
       </x:c>
       <x:c r="G244" s="23" t="n">
-        <x:v>69</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="H244" s="23" t="n">
         <x:v>74</x:v>
@@ -10120,7 +10120,7 @@
       <x:c r="K244" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L244" s="22"/>
+      <x:c r="L244" s="22" t="str"/>
       <x:c r="M244" s="24" t="str">
         <x:v>sbl_beer_10</x:v>
       </x:c>
@@ -10159,7 +10159,7 @@
       <x:c r="K245" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L245" s="22"/>
+      <x:c r="L245" s="22" t="str"/>
       <x:c r="M245" s="24" t="str">
         <x:v>sbl_beer_11</x:v>
       </x:c>
@@ -10198,7 +10198,7 @@
       <x:c r="K246" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L246" s="22"/>
+      <x:c r="L246" s="22" t="str"/>
       <x:c r="M246" s="24" t="str">
         <x:v>sbl_beer_12</x:v>
       </x:c>
@@ -10237,7 +10237,7 @@
       <x:c r="K247" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L247" s="22"/>
+      <x:c r="L247" s="22" t="str"/>
       <x:c r="M247" s="24" t="str">
         <x:v>sbl_beer_13</x:v>
       </x:c>
@@ -10303,7 +10303,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G249" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H249" s="23" t="n">
         <x:v>79</x:v>
@@ -10344,7 +10344,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G250" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="H250" s="23" t="n">
         <x:v>79</x:v>
@@ -10385,7 +10385,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G251" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="H251" s="23" t="n">
         <x:v>79</x:v>
@@ -10426,7 +10426,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G252" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="H252" s="23" t="n">
         <x:v>79</x:v>
@@ -10467,7 +10467,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G253" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H253" s="23" t="n">
         <x:v>79</x:v>
@@ -10508,7 +10508,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G254" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H254" s="23" t="n">
         <x:v>79</x:v>
@@ -10549,7 +10549,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G255" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H255" s="23" t="n">
         <x:v>77</x:v>
@@ -10563,7 +10563,7 @@
       <x:c r="K255" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L255" s="22"/>
+      <x:c r="L255" s="22" t="str"/>
       <x:c r="M255" s="24" t="str">
         <x:v>sbl_yulon_0</x:v>
       </x:c>
@@ -10588,7 +10588,7 @@
         <x:v>foreign</x:v>
       </x:c>
       <x:c r="G256" s="23" t="n">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H256" s="23" t="n">
         <x:v>87</x:v>
@@ -10602,7 +10602,7 @@
       <x:c r="K256" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L256" s="22"/>
+      <x:c r="L256" s="22" t="str"/>
       <x:c r="M256" s="24" t="str">
         <x:v>sbl_yulon_1</x:v>
       </x:c>
@@ -10641,7 +10641,7 @@
       <x:c r="K257" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L257" s="22"/>
+      <x:c r="L257" s="22" t="str"/>
       <x:c r="M257" s="24" t="str">
         <x:v>sbl_yulon_2</x:v>
       </x:c>
@@ -10680,7 +10680,7 @@
       <x:c r="K258" s="22" t="str">
         <x:v>提高團隊默契，降低比賽失誤波動。</x:v>
       </x:c>
-      <x:c r="L258" s="22"/>
+      <x:c r="L258" s="22" t="str"/>
       <x:c r="M258" s="24" t="str">
         <x:v>sbl_yulon_3</x:v>
       </x:c>
@@ -10719,7 +10719,7 @@
       <x:c r="K259" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L259" s="22"/>
+      <x:c r="L259" s="22" t="str"/>
       <x:c r="M259" s="24" t="str">
         <x:v>sbl_yulon_4</x:v>
       </x:c>
@@ -10744,7 +10744,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G260" s="23" t="n">
-        <x:v>74</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="H260" s="23" t="n">
         <x:v>79</x:v>
@@ -10758,7 +10758,7 @@
       <x:c r="K260" s="22" t="str">
         <x:v>空檔外線更穩定；快節奏戰術額外放大。</x:v>
       </x:c>
-      <x:c r="L260" s="22"/>
+      <x:c r="L260" s="22" t="str"/>
       <x:c r="M260" s="24" t="str">
         <x:v>sbl_yulon_5</x:v>
       </x:c>
@@ -10783,7 +10783,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G261" s="23" t="n">
-        <x:v>75</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="H261" s="23" t="n">
         <x:v>81</x:v>
@@ -10797,7 +10797,7 @@
       <x:c r="K261" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L261" s="22"/>
+      <x:c r="L261" s="22" t="str"/>
       <x:c r="M261" s="24" t="str">
         <x:v>sbl_yulon_6</x:v>
       </x:c>
@@ -10822,7 +10822,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G262" s="23" t="n">
-        <x:v>76</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="H262" s="23" t="n">
         <x:v>83</x:v>
@@ -10836,7 +10836,7 @@
       <x:c r="K262" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L262" s="22"/>
+      <x:c r="L262" s="22" t="str"/>
       <x:c r="M262" s="24" t="str">
         <x:v>sbl_yulon_7</x:v>
       </x:c>
@@ -10861,7 +10861,7 @@
         <x:v>local</x:v>
       </x:c>
       <x:c r="G263" s="23" t="n">
-        <x:v>77</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="H263" s="23" t="n">
         <x:v>85</x:v>
@@ -10875,7 +10875,7 @@
       <x:c r="K263" s="22" t="str">
         <x:v>攻守兩端都提供穩定的小幅加成。</x:v>
       </x:c>
-      <x:c r="L263" s="22"/>
+      <x:c r="L263" s="22" t="str"/>
       <x:c r="M263" s="24" t="str">
         <x:v>sbl_yulon_8</x:v>
       </x:c>
@@ -10914,7 +10914,7 @@
       <x:c r="K264" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L264" s="22"/>
+      <x:c r="L264" s="22" t="str"/>
       <x:c r="M264" s="24" t="str">
         <x:v>sbl_yulon_9</x:v>
       </x:c>
@@ -10953,7 +10953,7 @@
       <x:c r="K265" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L265" s="22"/>
+      <x:c r="L265" s="22" t="str"/>
       <x:c r="M265" s="24" t="str">
         <x:v>sbl_yulon_10</x:v>
       </x:c>
@@ -10992,7 +10992,7 @@
       <x:c r="K266" s="22" t="str">
         <x:v>擋拆與二次進攻更有效。</x:v>
       </x:c>
-      <x:c r="L266" s="22"/>
+      <x:c r="L266" s="22" t="str"/>
       <x:c r="M266" s="24" t="str">
         <x:v>sbl_yulon_11</x:v>
       </x:c>
@@ -11031,7 +11031,7 @@
       <x:c r="K267" s="22" t="str">
         <x:v>籃板回合更穩定，末節防守小幅提升。</x:v>
       </x:c>
-      <x:c r="L267" s="22"/>
+      <x:c r="L267" s="22" t="str"/>
       <x:c r="M267" s="24" t="str">
         <x:v>sbl_yulon_12</x:v>
       </x:c>
@@ -11040,7 +11040,7 @@
       <x:c r="A268" s="21" t="str">
         <x:v>公開資料補充</x:v>
       </x:c>
-      <x:c r="B268" s="22"/>
+      <x:c r="B268" s="22" t="str"/>
       <x:c r="C268" s="22" t="str">
         <x:v>謝宗融</x:v>
       </x:c>
@@ -11079,7 +11079,7 @@
       <x:c r="A269" s="21" t="str">
         <x:v>公開資料補充</x:v>
       </x:c>
-      <x:c r="B269" s="22"/>
+      <x:c r="B269" s="22" t="str"/>
       <x:c r="C269" s="22" t="str">
         <x:v>种義仁</x:v>
       </x:c>
@@ -11118,7 +11118,7 @@
       <x:c r="A270" s="21" t="str">
         <x:v>公開資料補充</x:v>
       </x:c>
-      <x:c r="B270" s="22"/>
+      <x:c r="B270" s="22" t="str"/>
       <x:c r="C270" s="22" t="str">
         <x:v>吳永盛</x:v>
       </x:c>
@@ -11157,7 +11157,7 @@
       <x:c r="A271" s="21" t="str">
         <x:v>公開資料補充</x:v>
       </x:c>
-      <x:c r="B271" s="22"/>
+      <x:c r="B271" s="22" t="str"/>
       <x:c r="C271" s="22" t="str">
         <x:v>郭少傑</x:v>
       </x:c>
@@ -11196,7 +11196,7 @@
       <x:c r="A272" s="21" t="str">
         <x:v>公開資料補充</x:v>
       </x:c>
-      <x:c r="B272" s="22"/>
+      <x:c r="B272" s="22" t="str"/>
       <x:c r="C272" s="22" t="str">
         <x:v>王律翔</x:v>
       </x:c>
@@ -11235,7 +11235,7 @@
       <x:c r="A273" s="21" t="str">
         <x:v>公開資料補充</x:v>
       </x:c>
-      <x:c r="B273" s="22"/>
+      <x:c r="B273" s="22" t="str"/>
       <x:c r="C273" s="22" t="str">
         <x:v>谷毛唯嘉</x:v>
       </x:c>
@@ -11274,7 +11274,7 @@
       <x:c r="A274" s="21" t="str">
         <x:v>公開資料補充</x:v>
       </x:c>
-      <x:c r="B274" s="22"/>
+      <x:c r="B274" s="22" t="str"/>
       <x:c r="C274" s="22" t="str">
         <x:v>李允傑</x:v>
       </x:c>
@@ -11313,7 +11313,7 @@
       <x:c r="A275" s="21" t="str">
         <x:v>公開資料補充</x:v>
       </x:c>
-      <x:c r="B275" s="22"/>
+      <x:c r="B275" s="22" t="str"/>
       <x:c r="C275" s="22" t="str">
         <x:v>陳力生</x:v>
       </x:c>
@@ -11352,7 +11352,7 @@
       <x:c r="A276" s="21" t="str">
         <x:v>公開資料補充</x:v>
       </x:c>
-      <x:c r="B276" s="22"/>
+      <x:c r="B276" s="22" t="str"/>
       <x:c r="C276" s="22" t="str">
         <x:v>張志豪</x:v>
       </x:c>
@@ -11391,7 +11391,7 @@
       <x:c r="A277" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B277" s="22"/>
+      <x:c r="B277" s="22" t="str"/>
       <x:c r="C277" s="22" t="str">
         <x:v>陳信安</x:v>
       </x:c>
@@ -11405,7 +11405,7 @@
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G277" s="23" t="n">
-        <x:v>82</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="H277" s="23" t="n">
         <x:v>0</x:v>
@@ -11419,14 +11419,14 @@
       <x:c r="K277" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L277" s="22"/>
-      <x:c r="M277" s="24"/>
+      <x:c r="L277" s="22" t="str"/>
+      <x:c r="M277" s="24" t="str"/>
     </x:row>
     <x:row r="278">
       <x:c r="A278" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B278" s="22"/>
+      <x:c r="B278" s="22" t="str"/>
       <x:c r="C278" s="22" t="str">
         <x:v>田壘</x:v>
       </x:c>
@@ -11454,14 +11454,14 @@
       <x:c r="K278" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L278" s="22"/>
-      <x:c r="M278" s="24"/>
+      <x:c r="L278" s="22" t="str"/>
+      <x:c r="M278" s="24" t="str"/>
     </x:row>
     <x:row r="279">
       <x:c r="A279" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B279" s="22"/>
+      <x:c r="B279" s="22" t="str"/>
       <x:c r="C279" s="22" t="str">
         <x:v>林志傑</x:v>
       </x:c>
@@ -11489,14 +11489,14 @@
       <x:c r="K279" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L279" s="22"/>
-      <x:c r="M279" s="24"/>
+      <x:c r="L279" s="22" t="str"/>
+      <x:c r="M279" s="24" t="str"/>
     </x:row>
     <x:row r="280">
       <x:c r="A280" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B280" s="22"/>
+      <x:c r="B280" s="22" t="str"/>
       <x:c r="C280" s="22" t="str">
         <x:v>戴維斯</x:v>
       </x:c>
@@ -11510,7 +11510,7 @@
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G280" s="23" t="n">
-        <x:v>79</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="H280" s="23" t="n">
         <x:v>0</x:v>
@@ -11524,14 +11524,14 @@
       <x:c r="K280" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L280" s="22"/>
-      <x:c r="M280" s="24"/>
+      <x:c r="L280" s="22" t="str"/>
+      <x:c r="M280" s="24" t="str"/>
     </x:row>
     <x:row r="281">
       <x:c r="A281" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B281" s="22"/>
+      <x:c r="B281" s="22" t="str"/>
       <x:c r="C281" s="22" t="str">
         <x:v>曾文鼎</x:v>
       </x:c>
@@ -11545,7 +11545,7 @@
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G281" s="23" t="n">
-        <x:v>78</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="H281" s="23" t="n">
         <x:v>0</x:v>
@@ -11559,14 +11559,14 @@
       <x:c r="K281" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L281" s="22"/>
-      <x:c r="M281" s="24"/>
+      <x:c r="L281" s="22" t="str"/>
+      <x:c r="M281" s="24" t="str"/>
     </x:row>
     <x:row r="282">
       <x:c r="A282" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B282" s="22"/>
+      <x:c r="B282" s="22" t="str"/>
       <x:c r="C282" s="22" t="str">
         <x:v>周儀翔</x:v>
       </x:c>
@@ -11594,14 +11594,14 @@
       <x:c r="K282" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L282" s="22"/>
-      <x:c r="M282" s="24"/>
+      <x:c r="L282" s="22" t="str"/>
+      <x:c r="M282" s="24" t="str"/>
     </x:row>
     <x:row r="283">
       <x:c r="A283" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B283" s="22"/>
+      <x:c r="B283" s="22" t="str"/>
       <x:c r="C283" s="22" t="str">
         <x:v>蔡文誠</x:v>
       </x:c>
@@ -11629,14 +11629,14 @@
       <x:c r="K283" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L283" s="22"/>
-      <x:c r="M283" s="24"/>
+      <x:c r="L283" s="22" t="str"/>
+      <x:c r="M283" s="24" t="str"/>
     </x:row>
     <x:row r="284">
       <x:c r="A284" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B284" s="22"/>
+      <x:c r="B284" s="22" t="str"/>
       <x:c r="C284" s="22" t="str">
         <x:v>楊敬敏</x:v>
       </x:c>
@@ -11650,7 +11650,7 @@
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G284" s="23" t="n">
-        <x:v>76</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H284" s="23" t="n">
         <x:v>0</x:v>
@@ -11664,14 +11664,14 @@
       <x:c r="K284" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L284" s="22"/>
-      <x:c r="M284" s="24"/>
+      <x:c r="L284" s="22" t="str"/>
+      <x:c r="M284" s="24" t="str"/>
     </x:row>
     <x:row r="285">
       <x:c r="A285" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B285" s="22"/>
+      <x:c r="B285" s="22" t="str"/>
       <x:c r="C285" s="22" t="str">
         <x:v>李學林</x:v>
       </x:c>
@@ -11685,7 +11685,7 @@
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G285" s="23" t="n">
-        <x:v>75</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="H285" s="23" t="n">
         <x:v>0</x:v>
@@ -11699,14 +11699,14 @@
       <x:c r="K285" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L285" s="22"/>
-      <x:c r="M285" s="24"/>
+      <x:c r="L285" s="22" t="str"/>
+      <x:c r="M285" s="24" t="str"/>
     </x:row>
     <x:row r="286">
       <x:c r="A286" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B286" s="22"/>
+      <x:c r="B286" s="22" t="str"/>
       <x:c r="C286" s="22" t="str">
         <x:v>吳岱豪</x:v>
       </x:c>
@@ -11734,14 +11734,14 @@
       <x:c r="K286" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L286" s="22"/>
-      <x:c r="M286" s="24"/>
+      <x:c r="L286" s="22" t="str"/>
+      <x:c r="M286" s="24" t="str"/>
     </x:row>
     <x:row r="287">
       <x:c r="A287" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B287" s="22"/>
+      <x:c r="B287" s="22" t="str"/>
       <x:c r="C287" s="22" t="str">
         <x:v>呂政儒</x:v>
       </x:c>
@@ -11769,14 +11769,14 @@
       <x:c r="K287" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L287" s="22"/>
-      <x:c r="M287" s="24"/>
+      <x:c r="L287" s="22" t="str"/>
+      <x:c r="M287" s="24" t="str"/>
     </x:row>
     <x:row r="288">
       <x:c r="A288" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B288" s="22"/>
+      <x:c r="B288" s="22" t="str"/>
       <x:c r="C288" s="22" t="str">
         <x:v>陳世念</x:v>
       </x:c>
@@ -11790,7 +11790,7 @@
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G288" s="23" t="n">
-        <x:v>73</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H288" s="23" t="n">
         <x:v>0</x:v>
@@ -11804,14 +11804,14 @@
       <x:c r="K288" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L288" s="22"/>
-      <x:c r="M288" s="24"/>
+      <x:c r="L288" s="22" t="str"/>
+      <x:c r="M288" s="24" t="str"/>
     </x:row>
     <x:row r="289">
       <x:c r="A289" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B289" s="22"/>
+      <x:c r="B289" s="22" t="str"/>
       <x:c r="C289" s="22" t="str">
         <x:v>簡浩</x:v>
       </x:c>
@@ -11825,7 +11825,7 @@
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G289" s="23" t="n">
-        <x:v>73</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="H289" s="23" t="n">
         <x:v>0</x:v>
@@ -11839,14 +11839,14 @@
       <x:c r="K289" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L289" s="22"/>
-      <x:c r="M289" s="24"/>
+      <x:c r="L289" s="22" t="str"/>
+      <x:c r="M289" s="24" t="str"/>
     </x:row>
     <x:row r="290">
       <x:c r="A290" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B290" s="22"/>
+      <x:c r="B290" s="22" t="str"/>
       <x:c r="C290" s="22" t="str">
         <x:v>周士淵</x:v>
       </x:c>
@@ -11860,7 +11860,7 @@
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G290" s="23" t="n">
-        <x:v>72</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H290" s="23" t="n">
         <x:v>0</x:v>
@@ -11874,14 +11874,14 @@
       <x:c r="K290" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L290" s="22"/>
-      <x:c r="M290" s="24"/>
+      <x:c r="L290" s="22" t="str"/>
+      <x:c r="M290" s="24" t="str"/>
     </x:row>
     <x:row r="291">
       <x:c r="A291" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B291" s="22"/>
+      <x:c r="B291" s="22" t="str"/>
       <x:c r="C291" s="22" t="str">
         <x:v>洪志善</x:v>
       </x:c>
@@ -11909,14 +11909,14 @@
       <x:c r="K291" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L291" s="22"/>
-      <x:c r="M291" s="24"/>
+      <x:c r="L291" s="22" t="str"/>
+      <x:c r="M291" s="24" t="str"/>
     </x:row>
     <x:row r="292">
       <x:c r="A292" s="21" t="str">
         <x:v>黃金世代老將</x:v>
       </x:c>
-      <x:c r="B292" s="22"/>
+      <x:c r="B292" s="22" t="str"/>
       <x:c r="C292" s="22" t="str">
         <x:v>吳永仁</x:v>
       </x:c>
@@ -11930,7 +11930,7 @@
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G292" s="23" t="n">
-        <x:v>70</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="H292" s="23" t="n">
         <x:v>0</x:v>
@@ -11944,8 +11944,8 @@
       <x:c r="K292" s="22" t="str">
         <x:v>提升年輕球員士氣，降低逆風默契損失。</x:v>
       </x:c>
-      <x:c r="L292" s="22"/>
-      <x:c r="M292" s="24"/>
+      <x:c r="L292" s="22" t="str"/>
+      <x:c r="M292" s="24" t="str"/>
     </x:row>
     <x:row r="293">
       <x:c r="A293" s="21" t="str">
@@ -11957,13 +11957,13 @@
       <x:c r="C293" s="22" t="str">
         <x:v>郭嘉安</x:v>
       </x:c>
-      <x:c r="D293" s="22"/>
-      <x:c r="E293" s="22"/>
+      <x:c r="D293" s="22" t="str"/>
+      <x:c r="E293" s="22" t="str"/>
       <x:c r="F293" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G293" s="23" t="n">
-        <x:v>68</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="H293" s="23" t="n">
         <x:v>0</x:v>
@@ -11977,7 +11977,7 @@
       <x:c r="K293" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L293" s="22"/>
+      <x:c r="L293" s="22" t="str"/>
       <x:c r="M293" s="24" t="str">
         <x:v>draft2026_郭嘉安</x:v>
       </x:c>
@@ -11992,8 +11992,8 @@
       <x:c r="C294" s="22" t="str">
         <x:v>史魯齊</x:v>
       </x:c>
-      <x:c r="D294" s="22"/>
-      <x:c r="E294" s="22"/>
+      <x:c r="D294" s="22" t="str"/>
+      <x:c r="E294" s="22" t="str"/>
       <x:c r="F294" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12012,7 +12012,7 @@
       <x:c r="K294" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L294" s="22"/>
+      <x:c r="L294" s="22" t="str"/>
       <x:c r="M294" s="24" t="str">
         <x:v>draft2026_史魯齊</x:v>
       </x:c>
@@ -12027,8 +12027,8 @@
       <x:c r="C295" s="22" t="str">
         <x:v>王語烽</x:v>
       </x:c>
-      <x:c r="D295" s="22"/>
-      <x:c r="E295" s="22"/>
+      <x:c r="D295" s="22" t="str"/>
+      <x:c r="E295" s="22" t="str"/>
       <x:c r="F295" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12047,7 +12047,7 @@
       <x:c r="K295" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L295" s="22"/>
+      <x:c r="L295" s="22" t="str"/>
       <x:c r="M295" s="24" t="str">
         <x:v>draft2026_王語烽</x:v>
       </x:c>
@@ -12062,13 +12062,13 @@
       <x:c r="C296" s="22" t="str">
         <x:v>李盛新</x:v>
       </x:c>
-      <x:c r="D296" s="22"/>
-      <x:c r="E296" s="22"/>
+      <x:c r="D296" s="22" t="str"/>
+      <x:c r="E296" s="22" t="str"/>
       <x:c r="F296" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G296" s="23" t="n">
-        <x:v>68</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="H296" s="23" t="n">
         <x:v>0</x:v>
@@ -12082,7 +12082,7 @@
       <x:c r="K296" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L296" s="22"/>
+      <x:c r="L296" s="22" t="str"/>
       <x:c r="M296" s="24" t="str">
         <x:v>draft2026_李盛新</x:v>
       </x:c>
@@ -12097,8 +12097,8 @@
       <x:c r="C297" s="22" t="str">
         <x:v>李宗漢</x:v>
       </x:c>
-      <x:c r="D297" s="22"/>
-      <x:c r="E297" s="22"/>
+      <x:c r="D297" s="22" t="str"/>
+      <x:c r="E297" s="22" t="str"/>
       <x:c r="F297" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12117,7 +12117,7 @@
       <x:c r="K297" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L297" s="22"/>
+      <x:c r="L297" s="22" t="str"/>
       <x:c r="M297" s="24" t="str">
         <x:v>draft2026_李宗漢</x:v>
       </x:c>
@@ -12132,8 +12132,8 @@
       <x:c r="C298" s="22" t="str">
         <x:v>劉恩任</x:v>
       </x:c>
-      <x:c r="D298" s="22"/>
-      <x:c r="E298" s="22"/>
+      <x:c r="D298" s="22" t="str"/>
+      <x:c r="E298" s="22" t="str"/>
       <x:c r="F298" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12152,7 +12152,7 @@
       <x:c r="K298" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L298" s="22"/>
+      <x:c r="L298" s="22" t="str"/>
       <x:c r="M298" s="24" t="str">
         <x:v>draft2026_劉恩任</x:v>
       </x:c>
@@ -12167,8 +12167,8 @@
       <x:c r="C299" s="22" t="str">
         <x:v>王鼎鈞</x:v>
       </x:c>
-      <x:c r="D299" s="22"/>
-      <x:c r="E299" s="22"/>
+      <x:c r="D299" s="22" t="str"/>
+      <x:c r="E299" s="22" t="str"/>
       <x:c r="F299" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12187,7 +12187,7 @@
       <x:c r="K299" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L299" s="22"/>
+      <x:c r="L299" s="22" t="str"/>
       <x:c r="M299" s="24" t="str">
         <x:v>draft2026_王鼎鈞</x:v>
       </x:c>
@@ -12202,8 +12202,8 @@
       <x:c r="C300" s="22" t="str">
         <x:v>史密斯</x:v>
       </x:c>
-      <x:c r="D300" s="22"/>
-      <x:c r="E300" s="22"/>
+      <x:c r="D300" s="22" t="str"/>
+      <x:c r="E300" s="22" t="str"/>
       <x:c r="F300" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12222,7 +12222,7 @@
       <x:c r="K300" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L300" s="22"/>
+      <x:c r="L300" s="22" t="str"/>
       <x:c r="M300" s="24" t="str">
         <x:v>draft2026_史密斯</x:v>
       </x:c>
@@ -12237,8 +12237,8 @@
       <x:c r="C301" s="22" t="str">
         <x:v>許浩翔</x:v>
       </x:c>
-      <x:c r="D301" s="22"/>
-      <x:c r="E301" s="22"/>
+      <x:c r="D301" s="22" t="str"/>
+      <x:c r="E301" s="22" t="str"/>
       <x:c r="F301" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12257,7 +12257,7 @@
       <x:c r="K301" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L301" s="22"/>
+      <x:c r="L301" s="22" t="str"/>
       <x:c r="M301" s="24" t="str">
         <x:v>draft2026_許浩翔</x:v>
       </x:c>
@@ -12272,8 +12272,8 @@
       <x:c r="C302" s="22" t="str">
         <x:v>潘偉傑</x:v>
       </x:c>
-      <x:c r="D302" s="22"/>
-      <x:c r="E302" s="22"/>
+      <x:c r="D302" s="22" t="str"/>
+      <x:c r="E302" s="22" t="str"/>
       <x:c r="F302" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12292,7 +12292,7 @@
       <x:c r="K302" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L302" s="22"/>
+      <x:c r="L302" s="22" t="str"/>
       <x:c r="M302" s="24" t="str">
         <x:v>draft2026_潘偉傑</x:v>
       </x:c>
@@ -12307,8 +12307,8 @@
       <x:c r="C303" s="22" t="str">
         <x:v>馬友程</x:v>
       </x:c>
-      <x:c r="D303" s="22"/>
-      <x:c r="E303" s="22"/>
+      <x:c r="D303" s="22" t="str"/>
+      <x:c r="E303" s="22" t="str"/>
       <x:c r="F303" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12327,7 +12327,7 @@
       <x:c r="K303" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L303" s="22"/>
+      <x:c r="L303" s="22" t="str"/>
       <x:c r="M303" s="24" t="str">
         <x:v>draft2026_馬友程</x:v>
       </x:c>
@@ -12342,8 +12342,8 @@
       <x:c r="C304" s="22" t="str">
         <x:v>陳宇軒</x:v>
       </x:c>
-      <x:c r="D304" s="22"/>
-      <x:c r="E304" s="22"/>
+      <x:c r="D304" s="22" t="str"/>
+      <x:c r="E304" s="22" t="str"/>
       <x:c r="F304" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12362,7 +12362,7 @@
       <x:c r="K304" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L304" s="22"/>
+      <x:c r="L304" s="22" t="str"/>
       <x:c r="M304" s="24" t="str">
         <x:v>draft2026_陳宇軒</x:v>
       </x:c>
@@ -12377,8 +12377,8 @@
       <x:c r="C305" s="22" t="str">
         <x:v>許皓洋</x:v>
       </x:c>
-      <x:c r="D305" s="22"/>
-      <x:c r="E305" s="22"/>
+      <x:c r="D305" s="22" t="str"/>
+      <x:c r="E305" s="22" t="str"/>
       <x:c r="F305" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12397,7 +12397,7 @@
       <x:c r="K305" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L305" s="22"/>
+      <x:c r="L305" s="22" t="str"/>
       <x:c r="M305" s="24" t="str">
         <x:v>draft2026_許皓洋</x:v>
       </x:c>
@@ -12412,8 +12412,8 @@
       <x:c r="C306" s="22" t="str">
         <x:v>張志守</x:v>
       </x:c>
-      <x:c r="D306" s="22"/>
-      <x:c r="E306" s="22"/>
+      <x:c r="D306" s="22" t="str"/>
+      <x:c r="E306" s="22" t="str"/>
       <x:c r="F306" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12432,7 +12432,7 @@
       <x:c r="K306" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L306" s="22"/>
+      <x:c r="L306" s="22" t="str"/>
       <x:c r="M306" s="24" t="str">
         <x:v>draft2026_張志守</x:v>
       </x:c>
@@ -12447,8 +12447,8 @@
       <x:c r="C307" s="22" t="str">
         <x:v>傅友</x:v>
       </x:c>
-      <x:c r="D307" s="22"/>
-      <x:c r="E307" s="22"/>
+      <x:c r="D307" s="22" t="str"/>
+      <x:c r="E307" s="22" t="str"/>
       <x:c r="F307" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12467,7 +12467,7 @@
       <x:c r="K307" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L307" s="22"/>
+      <x:c r="L307" s="22" t="str"/>
       <x:c r="M307" s="24" t="str">
         <x:v>draft2026_傅友</x:v>
       </x:c>
@@ -12482,8 +12482,8 @@
       <x:c r="C308" s="22" t="str">
         <x:v>張庭瑋</x:v>
       </x:c>
-      <x:c r="D308" s="22"/>
-      <x:c r="E308" s="22"/>
+      <x:c r="D308" s="22" t="str"/>
+      <x:c r="E308" s="22" t="str"/>
       <x:c r="F308" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12502,7 +12502,7 @@
       <x:c r="K308" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L308" s="22"/>
+      <x:c r="L308" s="22" t="str"/>
       <x:c r="M308" s="24" t="str">
         <x:v>draft2026_張庭瑋</x:v>
       </x:c>
@@ -12517,8 +12517,8 @@
       <x:c r="C309" s="22" t="str">
         <x:v>黃浚倢</x:v>
       </x:c>
-      <x:c r="D309" s="22"/>
-      <x:c r="E309" s="22"/>
+      <x:c r="D309" s="22" t="str"/>
+      <x:c r="E309" s="22" t="str"/>
       <x:c r="F309" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12537,7 +12537,7 @@
       <x:c r="K309" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L309" s="22"/>
+      <x:c r="L309" s="22" t="str"/>
       <x:c r="M309" s="24" t="str">
         <x:v>draft2026_黃浚倢</x:v>
       </x:c>
@@ -12552,8 +12552,8 @@
       <x:c r="C310" s="22" t="str">
         <x:v>陳柏丞</x:v>
       </x:c>
-      <x:c r="D310" s="22"/>
-      <x:c r="E310" s="22"/>
+      <x:c r="D310" s="22" t="str"/>
+      <x:c r="E310" s="22" t="str"/>
       <x:c r="F310" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12572,7 +12572,7 @@
       <x:c r="K310" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L310" s="22"/>
+      <x:c r="L310" s="22" t="str"/>
       <x:c r="M310" s="24" t="str">
         <x:v>draft2026_陳柏丞</x:v>
       </x:c>
@@ -12587,8 +12587,8 @@
       <x:c r="C311" s="22" t="str">
         <x:v>鄭文傑</x:v>
       </x:c>
-      <x:c r="D311" s="22"/>
-      <x:c r="E311" s="22"/>
+      <x:c r="D311" s="22" t="str"/>
+      <x:c r="E311" s="22" t="str"/>
       <x:c r="F311" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12607,7 +12607,7 @@
       <x:c r="K311" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L311" s="22"/>
+      <x:c r="L311" s="22" t="str"/>
       <x:c r="M311" s="24" t="str">
         <x:v>draft2026_鄭文傑</x:v>
       </x:c>
@@ -12622,8 +12622,8 @@
       <x:c r="C312" s="22" t="str">
         <x:v>莫森</x:v>
       </x:c>
-      <x:c r="D312" s="22"/>
-      <x:c r="E312" s="22"/>
+      <x:c r="D312" s="22" t="str"/>
+      <x:c r="E312" s="22" t="str"/>
       <x:c r="F312" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12642,7 +12642,7 @@
       <x:c r="K312" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L312" s="22"/>
+      <x:c r="L312" s="22" t="str"/>
       <x:c r="M312" s="24" t="str">
         <x:v>draft2026_莫森</x:v>
       </x:c>
@@ -12657,8 +12657,8 @@
       <x:c r="C313" s="22" t="str">
         <x:v>邱晨洋</x:v>
       </x:c>
-      <x:c r="D313" s="22"/>
-      <x:c r="E313" s="22"/>
+      <x:c r="D313" s="22" t="str"/>
+      <x:c r="E313" s="22" t="str"/>
       <x:c r="F313" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12677,7 +12677,7 @@
       <x:c r="K313" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L313" s="22"/>
+      <x:c r="L313" s="22" t="str"/>
       <x:c r="M313" s="24" t="str">
         <x:v>draft2026_邱晨洋</x:v>
       </x:c>
@@ -12692,13 +12692,13 @@
       <x:c r="C314" s="22" t="str">
         <x:v>吳志鍇</x:v>
       </x:c>
-      <x:c r="D314" s="22"/>
-      <x:c r="E314" s="22"/>
+      <x:c r="D314" s="22" t="str"/>
+      <x:c r="E314" s="22" t="str"/>
       <x:c r="F314" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G314" s="23" t="n">
-        <x:v>68</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="H314" s="23" t="n">
         <x:v>0</x:v>
@@ -12712,7 +12712,7 @@
       <x:c r="K314" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L314" s="22"/>
+      <x:c r="L314" s="22" t="str"/>
       <x:c r="M314" s="24" t="str">
         <x:v>draft2026_吳志鍇</x:v>
       </x:c>
@@ -12727,13 +12727,13 @@
       <x:c r="C315" s="22" t="str">
         <x:v>波波卡</x:v>
       </x:c>
-      <x:c r="D315" s="22"/>
-      <x:c r="E315" s="22"/>
+      <x:c r="D315" s="22" t="str"/>
+      <x:c r="E315" s="22" t="str"/>
       <x:c r="F315" s="22" t="str">
-        <x:v>本土</x:v>
+        <x:v>foreign_student-</x:v>
       </x:c>
       <x:c r="G315" s="23" t="n">
-        <x:v>68</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="H315" s="23" t="n">
         <x:v>0</x:v>
@@ -12747,7 +12747,7 @@
       <x:c r="K315" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L315" s="22"/>
+      <x:c r="L315" s="22" t="str"/>
       <x:c r="M315" s="24" t="str">
         <x:v>draft2026_波波卡</x:v>
       </x:c>
@@ -12762,8 +12762,8 @@
       <x:c r="C316" s="22" t="str">
         <x:v>林子桓</x:v>
       </x:c>
-      <x:c r="D316" s="22"/>
-      <x:c r="E316" s="22"/>
+      <x:c r="D316" s="22" t="str"/>
+      <x:c r="E316" s="22" t="str"/>
       <x:c r="F316" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12782,7 +12782,7 @@
       <x:c r="K316" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L316" s="22"/>
+      <x:c r="L316" s="22" t="str"/>
       <x:c r="M316" s="24" t="str">
         <x:v>draft2026_林子桓</x:v>
       </x:c>
@@ -12797,8 +12797,8 @@
       <x:c r="C317" s="22" t="str">
         <x:v>曾唯庭</x:v>
       </x:c>
-      <x:c r="D317" s="22"/>
-      <x:c r="E317" s="22"/>
+      <x:c r="D317" s="22" t="str"/>
+      <x:c r="E317" s="22" t="str"/>
       <x:c r="F317" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12817,7 +12817,7 @@
       <x:c r="K317" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L317" s="22"/>
+      <x:c r="L317" s="22" t="str"/>
       <x:c r="M317" s="24" t="str">
         <x:v>draft2026_曾唯庭</x:v>
       </x:c>
@@ -12832,13 +12832,13 @@
       <x:c r="C318" s="22" t="str">
         <x:v>賀丹</x:v>
       </x:c>
-      <x:c r="D318" s="22"/>
-      <x:c r="E318" s="22"/>
+      <x:c r="D318" s="22" t="str"/>
+      <x:c r="E318" s="22" t="str"/>
       <x:c r="F318" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
       <x:c r="G318" s="23" t="n">
-        <x:v>68</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="H318" s="23" t="n">
         <x:v>0</x:v>
@@ -12852,7 +12852,7 @@
       <x:c r="K318" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L318" s="22"/>
+      <x:c r="L318" s="22" t="str"/>
       <x:c r="M318" s="24" t="str">
         <x:v>draft2026_賀丹</x:v>
       </x:c>
@@ -12867,8 +12867,8 @@
       <x:c r="C319" s="22" t="str">
         <x:v>王俊凱</x:v>
       </x:c>
-      <x:c r="D319" s="22"/>
-      <x:c r="E319" s="22"/>
+      <x:c r="D319" s="22" t="str"/>
+      <x:c r="E319" s="22" t="str"/>
       <x:c r="F319" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12887,7 +12887,7 @@
       <x:c r="K319" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L319" s="22"/>
+      <x:c r="L319" s="22" t="str"/>
       <x:c r="M319" s="24" t="str">
         <x:v>draft2026_王俊凱</x:v>
       </x:c>
@@ -12902,8 +12902,8 @@
       <x:c r="C320" s="22" t="str">
         <x:v>蔡明峻</x:v>
       </x:c>
-      <x:c r="D320" s="22"/>
-      <x:c r="E320" s="22"/>
+      <x:c r="D320" s="22" t="str"/>
+      <x:c r="E320" s="22" t="str"/>
       <x:c r="F320" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12922,7 +12922,7 @@
       <x:c r="K320" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L320" s="22"/>
+      <x:c r="L320" s="22" t="str"/>
       <x:c r="M320" s="24" t="str">
         <x:v>draft2026_蔡明峻</x:v>
       </x:c>
@@ -12937,8 +12937,8 @@
       <x:c r="C321" s="22" t="str">
         <x:v>盧奕辰</x:v>
       </x:c>
-      <x:c r="D321" s="22"/>
-      <x:c r="E321" s="22"/>
+      <x:c r="D321" s="22" t="str"/>
+      <x:c r="E321" s="22" t="str"/>
       <x:c r="F321" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12957,7 +12957,7 @@
       <x:c r="K321" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L321" s="22"/>
+      <x:c r="L321" s="22" t="str"/>
       <x:c r="M321" s="24" t="str">
         <x:v>draft2026_盧奕辰</x:v>
       </x:c>
@@ -12972,8 +12972,8 @@
       <x:c r="C322" s="22" t="str">
         <x:v>李祐哲</x:v>
       </x:c>
-      <x:c r="D322" s="22"/>
-      <x:c r="E322" s="22"/>
+      <x:c r="D322" s="22" t="str"/>
+      <x:c r="E322" s="22" t="str"/>
       <x:c r="F322" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -12992,7 +12992,7 @@
       <x:c r="K322" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L322" s="22"/>
+      <x:c r="L322" s="22" t="str"/>
       <x:c r="M322" s="24" t="str">
         <x:v>draft2026_李祐哲</x:v>
       </x:c>
@@ -13007,8 +13007,8 @@
       <x:c r="C323" s="22" t="str">
         <x:v>陳恩</x:v>
       </x:c>
-      <x:c r="D323" s="22"/>
-      <x:c r="E323" s="22"/>
+      <x:c r="D323" s="22" t="str"/>
+      <x:c r="E323" s="22" t="str"/>
       <x:c r="F323" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13027,7 +13027,7 @@
       <x:c r="K323" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L323" s="22"/>
+      <x:c r="L323" s="22" t="str"/>
       <x:c r="M323" s="24" t="str">
         <x:v>draft2026_陳恩</x:v>
       </x:c>
@@ -13042,8 +13042,8 @@
       <x:c r="C324" s="22" t="str">
         <x:v>林瑞安</x:v>
       </x:c>
-      <x:c r="D324" s="22"/>
-      <x:c r="E324" s="22"/>
+      <x:c r="D324" s="22" t="str"/>
+      <x:c r="E324" s="22" t="str"/>
       <x:c r="F324" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13062,7 +13062,7 @@
       <x:c r="K324" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L324" s="22"/>
+      <x:c r="L324" s="22" t="str"/>
       <x:c r="M324" s="24" t="str">
         <x:v>draft2026_林瑞安</x:v>
       </x:c>
@@ -13077,8 +13077,8 @@
       <x:c r="C325" s="22" t="str">
         <x:v>廖胤辰</x:v>
       </x:c>
-      <x:c r="D325" s="22"/>
-      <x:c r="E325" s="22"/>
+      <x:c r="D325" s="22" t="str"/>
+      <x:c r="E325" s="22" t="str"/>
       <x:c r="F325" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13097,7 +13097,7 @@
       <x:c r="K325" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L325" s="22"/>
+      <x:c r="L325" s="22" t="str"/>
       <x:c r="M325" s="24" t="str">
         <x:v>draft2026_廖胤辰</x:v>
       </x:c>
@@ -13112,8 +13112,8 @@
       <x:c r="C326" s="22" t="str">
         <x:v>潘建宏</x:v>
       </x:c>
-      <x:c r="D326" s="22"/>
-      <x:c r="E326" s="22"/>
+      <x:c r="D326" s="22" t="str"/>
+      <x:c r="E326" s="22" t="str"/>
       <x:c r="F326" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13132,7 +13132,7 @@
       <x:c r="K326" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L326" s="22"/>
+      <x:c r="L326" s="22" t="str"/>
       <x:c r="M326" s="24" t="str">
         <x:v>draft2026_潘建宏</x:v>
       </x:c>
@@ -13147,8 +13147,8 @@
       <x:c r="C327" s="22" t="str">
         <x:v>陳廷霖</x:v>
       </x:c>
-      <x:c r="D327" s="22"/>
-      <x:c r="E327" s="22"/>
+      <x:c r="D327" s="22" t="str"/>
+      <x:c r="E327" s="22" t="str"/>
       <x:c r="F327" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13167,7 +13167,7 @@
       <x:c r="K327" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L327" s="22"/>
+      <x:c r="L327" s="22" t="str"/>
       <x:c r="M327" s="24" t="str">
         <x:v>draft2026_陳廷霖</x:v>
       </x:c>
@@ -13182,8 +13182,8 @@
       <x:c r="C328" s="22" t="str">
         <x:v>陳皓宇</x:v>
       </x:c>
-      <x:c r="D328" s="22"/>
-      <x:c r="E328" s="22"/>
+      <x:c r="D328" s="22" t="str"/>
+      <x:c r="E328" s="22" t="str"/>
       <x:c r="F328" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13202,7 +13202,7 @@
       <x:c r="K328" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L328" s="22"/>
+      <x:c r="L328" s="22" t="str"/>
       <x:c r="M328" s="24" t="str">
         <x:v>draft2026_陳皓宇</x:v>
       </x:c>
@@ -13217,8 +13217,8 @@
       <x:c r="C329" s="22" t="str">
         <x:v>潘彥愷</x:v>
       </x:c>
-      <x:c r="D329" s="22"/>
-      <x:c r="E329" s="22"/>
+      <x:c r="D329" s="22" t="str"/>
+      <x:c r="E329" s="22" t="str"/>
       <x:c r="F329" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13237,7 +13237,7 @@
       <x:c r="K329" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L329" s="22"/>
+      <x:c r="L329" s="22" t="str"/>
       <x:c r="M329" s="24" t="str">
         <x:v>draft2026_潘彥愷</x:v>
       </x:c>
@@ -13252,8 +13252,8 @@
       <x:c r="C330" s="22" t="str">
         <x:v>張東庭</x:v>
       </x:c>
-      <x:c r="D330" s="22"/>
-      <x:c r="E330" s="22"/>
+      <x:c r="D330" s="22" t="str"/>
+      <x:c r="E330" s="22" t="str"/>
       <x:c r="F330" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13272,7 +13272,7 @@
       <x:c r="K330" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L330" s="22"/>
+      <x:c r="L330" s="22" t="str"/>
       <x:c r="M330" s="24" t="str">
         <x:v>draft2026_張東庭</x:v>
       </x:c>
@@ -13287,10 +13287,10 @@
       <x:c r="C331" s="22" t="str">
         <x:v>莫斯塔發</x:v>
       </x:c>
-      <x:c r="D331" s="22"/>
-      <x:c r="E331" s="22"/>
+      <x:c r="D331" s="22" t="str"/>
+      <x:c r="E331" s="22" t="str"/>
       <x:c r="F331" s="22" t="str">
-        <x:v>本土</x:v>
+        <x:v>foreign_student</x:v>
       </x:c>
       <x:c r="G331" s="23" t="n">
         <x:v>68</x:v>
@@ -13307,7 +13307,7 @@
       <x:c r="K331" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L331" s="22"/>
+      <x:c r="L331" s="22" t="str"/>
       <x:c r="M331" s="24" t="str">
         <x:v>draft2026_莫斯塔發</x:v>
       </x:c>
@@ -13322,8 +13322,8 @@
       <x:c r="C332" s="22" t="str">
         <x:v>廖原祥</x:v>
       </x:c>
-      <x:c r="D332" s="22"/>
-      <x:c r="E332" s="22"/>
+      <x:c r="D332" s="22" t="str"/>
+      <x:c r="E332" s="22" t="str"/>
       <x:c r="F332" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13342,7 +13342,7 @@
       <x:c r="K332" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L332" s="22"/>
+      <x:c r="L332" s="22" t="str"/>
       <x:c r="M332" s="24" t="str">
         <x:v>draft2026_廖原祥</x:v>
       </x:c>
@@ -13357,8 +13357,8 @@
       <x:c r="C333" s="22" t="str">
         <x:v>蔡柏充</x:v>
       </x:c>
-      <x:c r="D333" s="22"/>
-      <x:c r="E333" s="22"/>
+      <x:c r="D333" s="22" t="str"/>
+      <x:c r="E333" s="22" t="str"/>
       <x:c r="F333" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13377,7 +13377,7 @@
       <x:c r="K333" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L333" s="22"/>
+      <x:c r="L333" s="22" t="str"/>
       <x:c r="M333" s="24" t="str">
         <x:v>draft2026_蔡柏充</x:v>
       </x:c>
@@ -13392,8 +13392,8 @@
       <x:c r="C334" s="22" t="str">
         <x:v>李書丞</x:v>
       </x:c>
-      <x:c r="D334" s="22"/>
-      <x:c r="E334" s="22"/>
+      <x:c r="D334" s="22" t="str"/>
+      <x:c r="E334" s="22" t="str"/>
       <x:c r="F334" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13412,7 +13412,7 @@
       <x:c r="K334" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L334" s="22"/>
+      <x:c r="L334" s="22" t="str"/>
       <x:c r="M334" s="24" t="str">
         <x:v>draft2026_李書丞</x:v>
       </x:c>
@@ -13427,8 +13427,8 @@
       <x:c r="C335" s="22" t="str">
         <x:v>杜帛鴻</x:v>
       </x:c>
-      <x:c r="D335" s="22"/>
-      <x:c r="E335" s="22"/>
+      <x:c r="D335" s="22" t="str"/>
+      <x:c r="E335" s="22" t="str"/>
       <x:c r="F335" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13447,7 +13447,7 @@
       <x:c r="K335" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L335" s="22"/>
+      <x:c r="L335" s="22" t="str"/>
       <x:c r="M335" s="24" t="str">
         <x:v>draft2026_杜帛鴻</x:v>
       </x:c>
@@ -13462,8 +13462,8 @@
       <x:c r="C336" s="22" t="str">
         <x:v>鞠丞哲</x:v>
       </x:c>
-      <x:c r="D336" s="22"/>
-      <x:c r="E336" s="22"/>
+      <x:c r="D336" s="22" t="str"/>
+      <x:c r="E336" s="22" t="str"/>
       <x:c r="F336" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13482,7 +13482,7 @@
       <x:c r="K336" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L336" s="22"/>
+      <x:c r="L336" s="22" t="str"/>
       <x:c r="M336" s="24" t="str">
         <x:v>draft2026_鞠丞哲</x:v>
       </x:c>
@@ -13497,8 +13497,8 @@
       <x:c r="C337" s="22" t="str">
         <x:v>劉皓瑋</x:v>
       </x:c>
-      <x:c r="D337" s="22"/>
-      <x:c r="E337" s="22"/>
+      <x:c r="D337" s="22" t="str"/>
+      <x:c r="E337" s="22" t="str"/>
       <x:c r="F337" s="22" t="str">
         <x:v>本土</x:v>
       </x:c>
@@ -13517,7 +13517,7 @@
       <x:c r="K337" s="22" t="str">
         <x:v>沒有特殊技能。</x:v>
       </x:c>
-      <x:c r="L337" s="22"/>
+      <x:c r="L337" s="22" t="str"/>
       <x:c r="M337" s="24" t="str">
         <x:v>draft2026_劉皓瑋</x:v>
       </x:c>
@@ -13600,7 +13600,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R514c9f9903e945f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f152798602f4f75"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>